<commit_message>
Texto completo: R0192 releído y excluido por CI-6; R0167 pendiente del PDF
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxN9W1XmdV2QxsHjBBQujW
</commit_message>
<xml_diff>
--- a/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
+++ b/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
@@ -230,10 +230,28 @@
 Motivo: Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
       </text>
     </comment>
+    <comment ref="E25" authorId="1" shapeId="0">
+      <text>
+        <t>Antes: Incluir
+Motivo: Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
+      </text>
+    </comment>
     <comment ref="F25" authorId="0" shapeId="0">
       <text>
         <t>Texto original:
 NO APLICA</t>
+      </text>
+    </comment>
+    <comment ref="G25" authorId="1" shapeId="0">
+      <text>
+        <t>Antes: El estudio propone SI-DMSeq, un modelo de Deep Learning multitarea basado en encoder-decoder LSTM con atención, para detectar anomalías de tráfico a nivel de red y de zonas (pp. 2-4, secciones I y III-A). La detección utiliza errores de reconstrucción, gráficos de control estadístico y puntuaciones locales mediante soft-thresholding (p. 7, sección III-F). Se valida con datos reales de Manhattan procedentes de aproximadamente 700 millones de viajes de taxi, agregados en 46 zonas (p. 8, sección IV
+Motivo: Cita del PDF.</t>
+      </text>
+    </comment>
+    <comment ref="H25" authorId="1" shapeId="0">
+      <text>
+        <t>Antes: [Incluir] Investigación original publicada en IEEE Access (2025), con texto completo Open Access. Presenta SI-DMSeq, arquitectura LSTM multitarea con atención que integra reconstrucción de secuencias, detección de anomalías e imputación de datos faltantes. Evalúa alteraciones del tráfico urbano a nivel global y local utilizando datos reales de Manhattan y dos eventos meteorológicos extremos. La detección se fundamenta en errores de reconstrucción y límites de control estadístico; la localización
+Motivo: Motivo.</t>
       </text>
     </comment>
     <comment ref="F30" authorId="0" shapeId="0">
@@ -5468,20 +5486,24 @@
           <t>cribado\pdf\R0192.pdf</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Incluir</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>El estudio propone SI-DMSeq, un modelo de Deep Learning multitarea basado en encoder-decoder LSTM con atención, para detectar anomalías de tráfico a nivel de red y de zonas (pp. 2-4, secciones I y III-A). La detección utiliza errores de reconstrucción, gráficos de control estadístico y puntuaciones locales mediante soft-thresholding (p. 7, sección III-F). Se valida con datos reales de Manhattan procedentes de aproximadamente 700 millones de viajes de taxi, agregados en 46 zonas (p. 8, sección IV-A). Identifica interrupciones durante el huracán Sandy y la tormenta de nieve de diciembre de 2010 (pp. 9-12). El modelo también realiza imputación de datos faltantes y presenta un tiempo medio de inferencia de 55 ms por secuencia (p. 12). Cumple los criterios de detección explícita de anomalías vehiculares mediante Deep Learning, validación empírica, periodo 2020-2026 y acceso abierto al texto completo.</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>[Incluir] Investigación original publicada en IEEE Access (2025), con texto completo Open Access. Presenta SI-DMSeq, arquitectura LSTM multitarea con atención que integra reconstrucción de secuencias, detección de anomalías e imputación de datos faltantes. Evalúa alteraciones del tráfico urbano a nivel global y local utilizando datos reales de Manhattan y dos eventos meteorológicos extremos. La detección se fundamenta en errores de reconstrucción y límites de control estadístico; la localización emplea puntuaciones de anomalía por zona. Los resultados respaldan la detección de interrupciones asociadas a eventos históricos. Limitaciones: evaluación restringida a Manhattan y eventos meteorológicos, validación principalmente gráfica de la detección y ausencia de métricas convencionales de clasificación como F1-score, precisión, recall y AUC. Cumple el objetivo de la revisión sistemática y pasa a extracción de datos y evaluación de calidad.</t>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Excluir</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>CI-6</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>"we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
         </is>
       </c>
     </row>
@@ -8570,7 +8592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8619,36 +8641,36 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>Paradigma no identificable («aprendizaje federado»): elegir una opción de la lista.</t>
+          <t>Paradigma no identificable («aprendizaje federado»): elegir una opción de la lista con el PDF (https://jcbi.org/index.php/Main/article/download/1147/825). Si el PDF ya no se puede obtener, poner DECISIÓN TC = «No recuperado».</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>R0192</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>REHACER</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>La hoja 2 está desplazada (cada valor en la columna equivocada): volver a pegar el bloque de 20 valores.</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>R0025</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Partición «No reportada» en la hoja 2 pero QA2 = 1 en la hoja 3: revisa uno de los dos.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>R0025</t>
+          <t>R0029</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -8663,14 +8685,14 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Partición «No reportada» en la hoja 2 pero QA2 = 1 en la hoja 3: revisa uno de los dos.</t>
+          <t>Se excluyó por CE-3 (clasifica perfiles normal/somnoliento/agresivo), pero R0032 (UAH-DriveSet, mismas tres clases), R0360, R0428 y R1029 se incluyeron. Decide con el mismo criterio para todos.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>R0029</t>
+          <t>R0051</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -8685,14 +8707,14 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Se excluyó por CE-3 (clasifica perfiles normal/somnoliento/agresivo), pero R0032 (UAH-DriveSet, mismas tres clases), R0360, R0428 y R1029 se incluyeron. Decide con el mismo criterio para todos.</t>
+          <t>Partición aleatoria (411/35/148) pero QA2 = 1: según la escala sería 0.5.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>R0051</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -8707,14 +8729,14 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Partición aleatoria (411/35/148) pero QA2 = 1: según la escala sería 0.5.</t>
+          <t>Caso límite: el DL extrae y reconstruye trayectorias y la anomalía se decide con reglas. Se mantiene incluido (regla de híbridos de CI-5); va al anexo de casos límite.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0986</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -8729,29 +8751,29 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Caso límite: el DL extrae y reconstruye trayectorias y la anomalía se decide con reglas. Se mantiene incluido (regla de híbridos de CI-5); va al anexo de casos límite.</t>
+          <t>El texto analizado corresponde a Systems and Soft Computing (DOI 10.1016/j.sasc.2025.200254), pero el registro tiene DOI 10.1002/spy2.70136: confirma que el PDF es el del registro.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>R0986</t>
+          <t>R0024</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Revisar</t>
+          <t>Corregido «QA8 Limitaciones» → 0</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>El texto analizado corresponde a Systems and Soft Computing (DOI 10.1016/j.sasc.2025.200254), pero el registro tiene DOI 10.1002/spy2.70136: confirma que el PDF es el del registro.</t>
+          <t>La hoja 2 dice «No reportadas»: la cita es trabajo futuro, no una limitación.</t>
         </is>
       </c>
     </row>
@@ -8768,41 +8790,41 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA8 Limitaciones» → 0</t>
+          <t>Corregido «QA8 evidencia» → No reportado (solo trabajo futuro, p. 10)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>La hoja 2 dice «No reportadas»: la cita es trabajo futuro, no una limitación.</t>
+          <t>Coherente con la hoja 2.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>R0024</t>
+          <t>R0032</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA8 evidencia» → No reportado (solo trabajo futuro, p. 10)</t>
+          <t>Corregido «Tipo de dato» → Multimodal</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Coherente con la hoja 2.</t>
+          <t>Acelerómetro, giroscopio y GPS del teléfono (UAH-DriveSet).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>R0032</t>
+          <t>R0052</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -8812,19 +8834,19 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Tipo de dato» → Multimodal</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Acelerómetro, giroscopio y GPS del teléfono (UAH-DriveSet).</t>
+          <t>Intersecciones y rampas/puentes de carretera.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>R0052</t>
+          <t>R0080</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -8834,19 +8856,19 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Intersecciones y rampas/puentes de carretera.</t>
+          <t>Incidentes distintos en entrenamiento (23) y prueba (22).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>R0080</t>
+          <t>R0097</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -8856,19 +8878,19 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Incidentes distintos en entrenamiento (23) y prueba (22).</t>
+          <t>Ubicación y tipo de vía no reportados.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>R0097</t>
+          <t>R0119</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -8878,12 +8900,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Ubicación y tipo de vía no reportados.</t>
+          <t>Intersecciones y autopistas.</t>
         </is>
       </c>
     </row>
@@ -8900,19 +8922,19 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «Partición» → Aleatoria</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Intersecciones y autopistas.</t>
+          <t>Partición estratificada sin separación temporal.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>R0119</t>
+          <t>R0121</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -8922,19 +8944,19 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «Entorno» → Urbano</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Partición estratificada sin separación temporal.</t>
+          <t>Dos cruces peatonales de calle (35 mph) en Florida.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>R0121</t>
+          <t>R0167</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -8944,19 +8966,19 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Urbano</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Dos cruces peatonales de calle (35 mph) en Florida.</t>
+          <t>«No se detallan particiones».</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>R0167</t>
+          <t>R0175</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -8966,19 +8988,19 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>«No se detallan particiones».</t>
+          <t>No especifica el tipo de vía.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>R0175</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -8988,41 +9010,41 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>No especifica el tipo de vía.</t>
+          <t>No describe la partición.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>R0185</t>
+          <t>R0190</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>No describe la partición.</t>
+          <t>Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>R0190</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -9032,19 +9054,19 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
+          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>R0244</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -9054,19 +9076,19 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Incluir</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>«INCLUIDO» no es una opción de la lista.</t>
+          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>R0249</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -9076,41 +9098,41 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>Cita del PDF.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>R0379</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Evalúa en una grabación highD no vista.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>R0389</t>
+          <t>R0244</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -9120,41 +9142,41 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «DECISIÓN TC» → Incluir</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
+          <t>«INCLUIDO» no es una opción de la lista.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0249</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA5 Código y datos» → 1</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
+          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0379</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -9169,80 +9191,80 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de DAD y CCD.</t>
+          <t>Evalúa en una grabación highD no vista.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0389</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Vías urbanas e interurbanas.</t>
+          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «QA5 Código y datos» → 1</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Conjunto externo ECVD solo para prueba.</t>
+          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>R0528</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
+          <t>Particiones oficiales de DAD y CCD.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>R0537</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -9252,19 +9274,19 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Sin proporciones ni protocolo de separación.</t>
+          <t>Vías urbanas e interurbanas.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>R0596</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -9274,41 +9296,41 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Partición insuficientemente reportada.</t>
+          <t>Conjunto externo ECVD solo para prueba.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>R0598</t>
+          <t>R0528</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Pista de pruebas; no es urbano ni autopista.</t>
+          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>R0601</t>
+          <t>R0537</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -9318,195 +9340,195 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de AI City Challenge.</t>
+          <t>Sin proporciones ni protocolo de separación.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0596</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
+          <t>Partición insuficientemente reportada.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0598</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Pista de pruebas; no es urbano ni autopista.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>R0614</t>
+          <t>R0601</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
+          <t>Conjunto de prueba de AI City Challenge.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>R0658</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de los benchmarks.</t>
+          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>R0664</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Videos de prueba separados.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0614</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>No detalla la partición.</t>
+          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0658</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
+          <t>Particiones oficiales de los benchmarks.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0664</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Videos de prueba separados.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>R0943</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -9521,58 +9543,58 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
+          <t>No detalla la partición.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>R1000</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>No indica qué escenas de NGSIM usa.</t>
+          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>R1010</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Evaluado con autos de juguete en escenario controlado.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>R1013</t>
+          <t>R0943</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -9582,19 +9604,19 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba oficial de TADS.</t>
+          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R1000</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -9604,19 +9626,19 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Familia DL principal» → Otra</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>DeepWalk/Node2vec no es una GNN.</t>
+          <t>No indica qué escenas de NGSIM usa.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>R1082</t>
+          <t>R1010</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -9626,19 +9648,19 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
+          <t>Evaluado con autos de juguete en escenario controlado.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>R1092</t>
+          <t>R1013</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -9648,19 +9670,19 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>División 80/20 de videos sin otro criterio.</t>
+          <t>Conjunto de prueba oficial de TADS.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>R1100</t>
+          <t>R1014</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -9670,19 +9692,19 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Familia DL principal» → Otra</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
+          <t>DeepWalk/Node2vec no es una GNN.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>R1138</t>
+          <t>R1082</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -9692,19 +9714,19 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>No desagrega urbano/autopista.</t>
+          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R1092</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -9714,19 +9736,19 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
+          <t>Corregido «Partición» → Aleatoria</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Objetos caídos sobre la calzada.</t>
+          <t>División 80/20 de videos sin otro criterio.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R1100</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -9736,41 +9758,41 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Solo dice que entrena y valida 100 épocas.</t>
+          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>R1166</t>
+          <t>R1138</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>No desagrega urbano/autopista.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>R1185</t>
+          <t>R1148</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -9780,19 +9802,19 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>No clasifica las imágenes por tipo de vía.</t>
+          <t>Objetos caídos sobre la calzada.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>R1202</t>
+          <t>R1148</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -9802,32 +9824,98 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Separación por sesiones de conducción.</t>
+          <t>Solo dice que entrena y valida 100 épocas.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
+          <t>R1166</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «CRITERIO» → CI-6</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>R1185</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>No clasifica las imágenes por tipo de vía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>R1202</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Separación por sesiones de conducción.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
           <t>R1214</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>No informa proporciones ni criterio de división.</t>
         </is>
@@ -12458,94 +12546,94 @@
       </c>
     </row>
     <row r="25" ht="28.8" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>R0192</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>A Self-Imputing Deep Multitask Sequence Model for Traffic Disruption Detection in Extreme Conditions</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>cribado\pdf\R0192.pdf</t>
         </is>
       </c>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>SI-DMSeq (Self-Imputing Deep Multitask Sequence)</t>
         </is>
       </c>
-      <c r="H25" s="9" t="n"/>
-      <c r="I25" s="9" t="inlineStr">
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>Encoder LSTM compartido y dos decodificadores LSTM con atención para reconstrucción y predicción</t>
         </is>
       </c>
-      <c r="J25" s="9" t="n"/>
-      <c r="K25" s="9" t="n"/>
-      <c r="L25" s="9" t="inlineStr">
+      <c r="J25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t>Manhattan, Nueva York, Estados Unidos</t>
         </is>
       </c>
-      <c r="M25" s="9" t="n"/>
-      <c r="N25" s="9" t="inlineStr">
+      <c r="M25" s="5" t="n"/>
+      <c r="N25" s="5" t="inlineStr">
         <is>
           <t>Evento/otro</t>
         </is>
       </c>
-      <c r="O25" s="9" t="inlineStr">
+      <c r="O25" s="5" t="inlineStr">
         <is>
           <t>Detección no supervisada basada en aprendizaje de patrones normales</t>
         </is>
       </c>
-      <c r="P25" s="9" t="inlineStr">
+      <c r="P25" s="5" t="inlineStr">
         <is>
           <t>Errores de reconstrucción MSE, gráficos de control estadístico SPC y soft-thresholding por zona</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
+      <c r="Q25" s="5" t="inlineStr">
         <is>
           <t>Detección a nivel de red y localización de zonas afectadas por eventos extremos</t>
         </is>
       </c>
-      <c r="R25" s="9" t="inlineStr">
+      <c r="R25" s="5" t="inlineStr">
         <is>
           <t>RMSE para imputación; estadístico MSE y límites de control para detección; validación visual de anomalías</t>
         </is>
       </c>
-      <c r="S25" s="9" t="inlineStr">
+      <c r="S25" s="5" t="inlineStr">
         <is>
           <t>Aleatoria</t>
         </is>
       </c>
-      <c r="T25" s="9" t="inlineStr">
+      <c r="T25" s="5" t="inlineStr">
         <is>
           <t>Comparación de imputación con Temporal Mean, RTRC y PARATUCK2</t>
         </is>
       </c>
-      <c r="U25" s="9" t="n"/>
-      <c r="V25" s="9" t="inlineStr">
+      <c r="U25" s="5" t="n"/>
+      <c r="V25" s="5" t="inlineStr">
         <is>
           <t>Detección de anomalías a dos escalas, imputación integrada y procesamiento apto para monitoreo casi en tiempo real</t>
         </is>
       </c>
-      <c r="W25" s="9" t="inlineStr">
+      <c r="W25" s="5" t="inlineStr">
         <is>
           <t>Evaluación limitada a Manhattan y eventos meteorológicos; validación de detección principalmente visual; sin precisión, recall, F1-score ni AUC reportados</t>
         </is>
       </c>
-      <c r="X25" s="9" t="inlineStr">
+      <c r="X25" s="5" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/ACCESS.2025.3612407 ; https://github.com/minanouri/SI-DMSeq</t>
         </is>

</xml_diff>

<commit_message>
Texto completo cerrado: 77 incluidos, 15 excluidos, 11 no recuperados; PRISMA y script de Parsif.al
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxN9W1XmdV2QxsHjBBQujW
</commit_message>
<xml_diff>
--- a/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
+++ b/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
@@ -42,7 +42,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,11 +81,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0000467F"/>
       </patternFill>
     </fill>
@@ -102,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -125,10 +120,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -208,473 +200,491 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
+    <author>Revisión</author>
     <author>Normalización</author>
-    <author>Revisión</author>
   </authors>
   <commentList>
-    <comment ref="F6" authorId="0" shapeId="0">
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Excluir
+Motivo: El autor verificó que no hay texto completo en acceso abierto (la copia de SSRN no está disponible).</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: CE-3
+Motivo: No recuperado no lleva criterio.</t>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: [Excluir CE-3] Estudio comparativo de clasificación de perfiles de conducción mediante ML, DL y ensamble PSO; no presenta una tarea específica de detección o anticipación de anomalías vehiculares.
+Motivo: Coherente con las demás no recuperadas.</t>
+      </text>
+    </comment>
+    <comment ref="F6" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de inclusión por ser un artículo original de conferencia ACM publicado en 2026, con texto completo disponible, aplicación a conducción vehicular real, modelos de Deep Learning y evaluación cuantitativa de comportamientos de riesgo. Se incluye como clasificación supervisada de conducción normal, agresiva y somnolienta, no como detección no supervisada de anomalías desconocidas.</t>
       </text>
     </comment>
-    <comment ref="F7" authorId="0" shapeId="0">
+    <comment ref="F7" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 —</t>
       </text>
     </comment>
-    <comment ref="F24" authorId="1" shapeId="0">
+    <comment ref="F24" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-2
 Motivo: Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
       </text>
     </comment>
-    <comment ref="E25" authorId="1" shapeId="0">
+    <comment ref="E25" authorId="0" shapeId="0">
       <text>
         <t>Antes: Incluir
 Motivo: Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
       </text>
     </comment>
-    <comment ref="F25" authorId="0" shapeId="0">
+    <comment ref="F25" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 NO APLICA</t>
       </text>
     </comment>
-    <comment ref="G25" authorId="1" shapeId="0">
+    <comment ref="G25" authorId="0" shapeId="0">
       <text>
         <t>Antes: El estudio propone SI-DMSeq, un modelo de Deep Learning multitarea basado en encoder-decoder LSTM con atención, para detectar anomalías de tráfico a nivel de red y de zonas (pp. 2-4, secciones I y III-A). La detección utiliza errores de reconstrucción, gráficos de control estadístico y puntuaciones locales mediante soft-thresholding (p. 7, sección III-F). Se valida con datos reales de Manhattan procedentes de aproximadamente 700 millones de viajes de taxi, agregados en 46 zonas (p. 8, sección IV
 Motivo: Cita del PDF.</t>
       </text>
     </comment>
-    <comment ref="H25" authorId="1" shapeId="0">
+    <comment ref="H25" authorId="0" shapeId="0">
       <text>
         <t>Antes: [Incluir] Investigación original publicada en IEEE Access (2025), con texto completo Open Access. Presenta SI-DMSeq, arquitectura LSTM multitarea con atención que integra reconstrucción de secuencias, detección de anomalías e imputación de datos faltantes. Evalúa alteraciones del tráfico urbano a nivel global y local utilizando datos reales de Manhattan y dos eventos meteorológicos extremos. La detección se fundamenta en errores de reconstrucción y límites de control estadístico; la localización
 Motivo: Motivo.</t>
       </text>
     </comment>
-    <comment ref="F30" authorId="0" shapeId="0">
+    <comment ref="F30" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 NO APLICA</t>
       </text>
     </comment>
-    <comment ref="F31" authorId="1" shapeId="0">
+    <comment ref="F31" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-3
 Motivo: Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
       </text>
     </comment>
-    <comment ref="F32" authorId="0" shapeId="0">
+    <comment ref="F32" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F33" authorId="0" shapeId="0">
+    <comment ref="F33" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión</t>
       </text>
     </comment>
-    <comment ref="F34" authorId="0" shapeId="0">
+    <comment ref="F34" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión</t>
       </text>
     </comment>
-    <comment ref="F36" authorId="0" shapeId="0">
+    <comment ref="F36" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F37" authorId="0" shapeId="0">
+    <comment ref="F37" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F38" authorId="0" shapeId="0">
+    <comment ref="F38" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F39" authorId="0" shapeId="0">
+    <comment ref="F39" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F40" authorId="0" shapeId="0">
+    <comment ref="F40" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F41" authorId="0" shapeId="0">
+    <comment ref="F41" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F42" authorId="1" shapeId="0">
+    <comment ref="F42" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-3
 Motivo: Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
       </text>
     </comment>
-    <comment ref="F43" authorId="0" shapeId="0">
+    <comment ref="F43" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de inclusión por ser un artículo original revisado por pares, publicado en 2025 y disponible en acceso abierto, que desarrolla y evalúa cuantitativamente un modelo de Deep Learning para anticipación de accidentes vehiculares. La tarea se considera detección anticipada de situaciones anormales de riesgo, no detección retrospectiva de accidentes.</t>
       </text>
     </comment>
-    <comment ref="F44" authorId="0" shapeId="0">
+    <comment ref="F44" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F45" authorId="0" shapeId="0">
+    <comment ref="F45" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F46" authorId="0" shapeId="0">
+    <comment ref="F46" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F47" authorId="0" shapeId="0">
+    <comment ref="F47" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F49" authorId="0" shapeId="0">
+    <comment ref="F49" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F51" authorId="1" shapeId="0">
+    <comment ref="F51" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-3
 Motivo: Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
       </text>
     </comment>
-    <comment ref="F52" authorId="0" shapeId="0">
+    <comment ref="F52" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F53" authorId="0" shapeId="0">
+    <comment ref="F53" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F54" authorId="0" shapeId="0">
+    <comment ref="F54" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F55" authorId="0" shapeId="0">
+    <comment ref="F55" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F56" authorId="0" shapeId="0">
+    <comment ref="F56" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F57" authorId="0" shapeId="0">
+    <comment ref="F57" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-5: Tipo de publicación no elegible; tesis de maestría, sin evidencia de publicación de este documento como artículo revisado por pares.</t>
       </text>
     </comment>
-    <comment ref="F59" authorId="0" shapeId="0">
+    <comment ref="F59" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión.</t>
       </text>
     </comment>
-    <comment ref="F60" authorId="0" shapeId="0">
+    <comment ref="F60" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión.</t>
       </text>
     </comment>
-    <comment ref="F61" authorId="0" shapeId="0">
+    <comment ref="F61" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios temáticos y de acceso, aunque presenta reservas importantes sobre la validez de los resultados.</t>
       </text>
     </comment>
-    <comment ref="F62" authorId="0" shapeId="0">
+    <comment ref="F62" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="E63" authorId="1" shapeId="0">
+    <comment ref="E63" authorId="0" shapeId="0">
       <text>
         <t>Antes: Incluir
 Motivo: Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
       </text>
     </comment>
-    <comment ref="F63" authorId="0" shapeId="0">
+    <comment ref="F63" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica</t>
       </text>
     </comment>
-    <comment ref="F64" authorId="1" shapeId="0">
+    <comment ref="F64" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-4
 Motivo: Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
       </text>
     </comment>
-    <comment ref="F65" authorId="0" shapeId="0">
+    <comment ref="F65" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica. Cumple los criterios de inclusión: artículo original de revista publicado en 2025; tráfico vehicular terrestre en carreteras montañosas; utilización de una red neuronal profunda LSTM; detección explícita de incidentes mediante clasificación binaria; evaluación cuantitativa con DR, FAR, F1, accuracy y AUC; texto completo accesible.</t>
       </text>
     </comment>
-    <comment ref="F66" authorId="0" shapeId="0">
+    <comment ref="F66" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-5: documento disponible como prepublicación arXiv, sin evidencia de publicación arbitrada en revista o congreso dentro del PDF. El manuscrito se identifica como arXiv:2505.02613v1, fechado el 5 de mayo de 2025, y no presenta DOI editorial, nombre de congreso, revista ni datos de aceptación. La exclusión se refiere al estado de publicación verificable de esta versión; no implica que el trabajo carezca de calidad científica ni descarta una eventual versión publicada posteriormente.</t>
       </text>
     </comment>
-    <comment ref="F67" authorId="0" shapeId="0">
+    <comment ref="F67" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-5: prepublicación arXiv sin acreditación de revisión por pares en la versión PDF examinada. El documento figura como arXiv:2303.05000v1 [cs.LG], fechado el 9 de marzo de 2023, sin nombre de revista, congreso, volumen, páginas editoriales ni DOI de publicación. La decisión corresponde exclusivamente a esta versión documental y deberá reconsiderarse si se identifica una publicación arbitrada equivalente.</t>
       </text>
     </comment>
-    <comment ref="F69" authorId="0" shapeId="0">
+    <comment ref="F69" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-3: El estudio se centra en predicción de riesgo de colisión y no demuestra un sistema de detección explícita de anomalías vehiculares en tráfico general. Aunque clasifica muestras peligrosas y presenta métricas de clasificación, los escenarios peligrosos se preseleccionan mediante TTC &lt; 3 s; el propio artículo reconoce que todavía es necesario identificar esos periodos en aplicaciones reales.</t>
       </text>
     </comment>
-    <comment ref="F70" authorId="0" shapeId="0">
+    <comment ref="F70" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión. Artículo original de revista publicado en 2020, dentro del intervalo 2020–2026, centrado en la identificación explícita de comportamientos anómalos de conducción vehicular mediante una arquitectura híbrida de Deep Learning LSTM-CNN, con datos reales y evaluación cuantitativa.</t>
       </text>
     </comment>
-    <comment ref="F71" authorId="0" shapeId="0">
+    <comment ref="F71" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-3: el estudio no evalúa cuantitativamente la detección de anomalías en tráfico vehicular. Aunque propone un modelo Deep Learning para analizar conducción peligrosa, su tarea experimental es la predicción de series temporales y del nivel macroscópico de riesgo generado mediante reglas difusas, sin contrastar decisiones de anomalía contra etiquetas de referencia independientes.</t>
       </text>
     </comment>
-    <comment ref="F72" authorId="0" shapeId="0">
+    <comment ref="F72" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión por tratarse de un artículo original de revista científica publicado en 2025, con texto completo disponible, uso de Deep Learning y evaluación cuantitativa de detección de anomalías en tráfico vehicular mediante UIT-ADrone.</t>
       </text>
     </comment>
-    <comment ref="F73" authorId="0" shapeId="0">
+    <comment ref="F73" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; cumple los criterios de inclusión por ser un artículo original de revista científica de 2025, con acceso abierto al texto completo, modelo basado en Deep Learning y evaluación cuantitativa de incidentes de tráfico vehicular.</t>
       </text>
     </comment>
-    <comment ref="F74" authorId="0" shapeId="0">
+    <comment ref="F74" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; artículo original de revista científica, publicado en 2024, con texto completo abierto y evaluación cuantitativa de comportamientos anómalos en autopistas mediante un sistema que incorpora redes profundas. La inclusión es condicionada a que el protocolo acepte Deep Learning para obtener y reconstruir trayectorias, aunque la decisión final de anomalía se base en reglas.</t>
       </text>
     </comment>
-    <comment ref="F75" authorId="0" shapeId="0">
+    <comment ref="F75" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; estudio original publicado en una conferencia científica ACM KDD 2024, dentro del periodo 2020–2026, con texto completo disponible, aplicación explícita de Deep Learning y evaluación cuantitativa de detección de trayectorias vehiculares anómalas.</t>
       </text>
     </comment>
-    <comment ref="F76" authorId="0" shapeId="0">
+    <comment ref="F76" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; artículo original publicado en Scientific Reports, volumen 16, artículo 1516, año 2026, con texto completo Open Access. Aborda tráfico vehicular terrestre, utiliza aprendizaje profundo mediante atención multi-head y LSTM, y presenta evaluación cuantitativa de detección de anomalías e identificación de incidentes.</t>
       </text>
     </comment>
-    <comment ref="F77" authorId="0" shapeId="0">
+    <comment ref="F77" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; estudio original de conferencia científica IEEE ICDE 2023, dentro del periodo 2020–2026, con texto completo disponible. Analiza trayectorias reales de taxis sobre redes viales y propone un modelo de Deep Reinforcement Learning para detectar y localizar subtrayectorias anómalas en línea, con evaluación cuantitativa mediante F1 y TF1.</t>
       </text>
     </comment>
-    <comment ref="F78" authorId="0" shapeId="0">
+    <comment ref="F78" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; artículo científico original publicado en 2023, dentro del periodo 2020–2026, con texto completo accesible. Aborda detección explícita de trayectorias anómalas de vehículos terrestres mediante aprendizaje profundo recurrente y reporta resultados cuantitativos de detección sobre dos conjuntos de datos reales.</t>
       </text>
     </comment>
-    <comment ref="E79" authorId="1" shapeId="0">
+    <comment ref="E79" authorId="0" shapeId="0">
       <text>
         <t>Antes: Incluir
 Motivo: La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
       </text>
     </comment>
-    <comment ref="F79" authorId="0" shapeId="0">
+    <comment ref="F79" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; estudio original publicado en una conferencia ACM de 2024, con texto completo disponible. Desarrolla y evalúa una CNN para reconocer una conducta anómala de conducción, específicamente el uso del teléfono móvil, y la integra en un sistema de seguridad vehicular.</t>
       </text>
     </comment>
-    <comment ref="F80" authorId="0" shapeId="0">
+    <comment ref="F80" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; artículo original de investigación publicado en Heliyon en 2025, dentro del periodo 2020–2026, con texto completo Open Access. Estudia explícitamente la detección de accidentes en tráfico vehicular terrestre mediante modelos de Deep Learning y presenta métricas cuantitativas de detección.</t>
       </text>
     </comment>
-    <comment ref="F81" authorId="0" shapeId="0">
+    <comment ref="F81" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; estudio original publicado en Transportation Research Procedia, volumen 85, páginas 68–75, en 2025, con revisión por pares y texto completo Open Access. Investiga explícitamente la detección de accidentes vehiculares terrestres mediante Deep Learning y presenta métricas cuantitativas de detección.</t>
       </text>
     </comment>
-    <comment ref="F82" authorId="0" shapeId="0">
+    <comment ref="F82" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; artículo original de revista científica publicado en Chinese Journal of Mechanical Engineering, volumen 39 (2026), artículo 100169, DOI 10.1016/j.cjme.2025.100169, con texto completo Open Access bajo licencia CC BY 4.0. Se encuentra dentro del periodo 2020–2026, estudia tráfico vehicular terrestre, desarrolla un modelo de Deep Learning y evalúa cuantitativamente la detección de comportamientos de conducción anómalos.</t>
       </text>
     </comment>
-    <comment ref="F83" authorId="0" shapeId="0">
+    <comment ref="F83" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-3 — El estudio no desarrolla ni evalúa cuantitativamente un método de detección de anomalías en tráfico vehicular. Su objetivo principal es la predicción no lineal del flujo de tráfico mediante una red LSTM de dos capas y una infraestructura IoT. Aunque menciona incidentes, condiciones anormales, valores atípicos y fallos de sensores, no presenta etiquetas de anomalías viales, una regla de clasificación de eventos anómalos ni métricas específicas de detección.</t>
       </text>
     </comment>
-    <comment ref="F84" authorId="0" shapeId="0">
+    <comment ref="F84" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — El estudio cumple los criterios de inclusión: artículo científico original de revista, publicado dentro del periodo 2020–2026, texto completo Open Access, tráfico vehicular terrestre, modelo basado en Deep Learning y evaluación cuantitativa explícita de detección de anomalías.</t>
       </text>
     </comment>
-    <comment ref="F85" authorId="0" shapeId="0">
+    <comment ref="F85" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo original de conferencia ACM publicado en 2025, con texto completo Open Access; aborda incidentes de tráfico vehicular mediante Deep Learning y presenta evaluación cuantitativa de detección de accidentes.</t>
       </text>
     </comment>
-    <comment ref="F86" authorId="0" shapeId="0">
+    <comment ref="F86" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Estudio original publicado en Sensors en 2026, con revisión por pares y texto completo Open Access; desarrolla y evalúa cuantitativamente un modelo de Deep Learning para detectar accidentes y anomalías del tráfico vehicular mediante videos de vigilancia.</t>
       </text>
     </comment>
-    <comment ref="F87" authorId="0" shapeId="0">
+    <comment ref="F87" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo original de investigación publicado en revista científica, dentro del periodo 2020–2026, con texto completo Open Access; aborda explícitamente la detección de trayectorias anómalas y regiones de tráfico vehicular anormal mediante aprendizaje neuronal de representaciones de grafos.</t>
       </text>
     </comment>
-    <comment ref="F88" authorId="0" shapeId="0">
+    <comment ref="F88" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Estudio original publicado en revista científica revisada por pares en 2026, con texto completo Open Access, que aborda explícitamente la detección de comportamiento anómalo de conducción mediante redes neuronales profundas y reporta métricas cuantitativas de clasificación.</t>
       </text>
     </comment>
-    <comment ref="F89" authorId="0" shapeId="0">
+    <comment ref="F89" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo original publicado en revista científica en 2026, con acceso abierto y aplicación explícita de Deep Learning a la detección y clasificación de incidentes de tráfico vehicular.</t>
       </text>
     </comment>
-    <comment ref="F90" authorId="0" shapeId="0">
+    <comment ref="F90" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Estudio original revisado por pares, publicado en IEEE Access en 2024, con texto completo accesible; desarrolla y evalúa un modelo de Deep Learning para detectar accidentes vehiculares mediante video.</t>
       </text>
     </comment>
-    <comment ref="F91" authorId="0" shapeId="0">
+    <comment ref="F91" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo científico original publicado en Sensors en 2023, dentro del periodo 2020–2026, revisado por pares y disponible en acceso abierto. Aborda directamente la identificación de eventos extraordinarios del tráfico vehicular mediante redes neuronales profundas y presenta evaluación cuantitativa sobre imágenes reales de autopistas.</t>
       </text>
     </comment>
-    <comment ref="F92" authorId="0" shapeId="0">
+    <comment ref="F92" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Estudio original publicado en las actas de AAMAS 2023, dentro del periodo 2020–2026, con texto completo accesible gratuitamente. Investiga directamente la detección de anomalías en tráfico vehicular de autopista mediante Deep Learning y reporta resultados cuantitativos de detección.</t>
       </text>
     </comment>
-    <comment ref="F93" authorId="0" shapeId="0">
+    <comment ref="F93" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo original publicado en Scientific Reports en 2026, dentro del periodo 2020–2026, con texto completo de acceso abierto. Presenta una arquitectura basada en redes neuronales convolucionales para detectar y clasificar anomalías en tráfico vehicular mediante videos de vigilancia aérea y ofrece evaluación cuantitativa.</t>
       </text>
     </comment>
-    <comment ref="F94" authorId="0" shapeId="0">
+    <comment ref="F94" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo original de revista científica publicado en 2026, dentro del periodo de la revisión. Emplea Deep Learning y presenta una tarea explícita de detección de accidentes de tráfico con evaluación cuantitativa. El PDF completo está disponible para análisis.</t>
       </text>
     </comment>
-    <comment ref="F95" authorId="0" shapeId="0">
+    <comment ref="F95" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Estudio original publicado en IEEE Access en diciembre de 2023, dentro del periodo 2020–2026; artículo revisado por pares, con texto completo de acceso abierto, modelo de Deep Learning y evaluación cuantitativa explícita de detección de accidentes de tráfico.</t>
       </text>
     </comment>
-    <comment ref="F96" authorId="0" shapeId="0">
+    <comment ref="F96" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de elegibilidad; es un artículo científico original publicado en Mathematics en 2023, con texto completo de acceso abierto, aplicación explícita de Deep Learning al tráfico vehicular terrestre y evaluación cuantitativa de la detección de accidentes.</t>
       </text>
     </comment>
-    <comment ref="F97" authorId="0" shapeId="0">
+    <comment ref="F97" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: artículo original revisado por pares, publicado en Mathematics en 2023, con texto completo de acceso abierto, aplicación explícita de Deep Learning al tráfico vehicular terrestre y evaluación cuantitativa de detección de accidentes.</t>
       </text>
     </comment>
-    <comment ref="F99" authorId="0" shapeId="0">
+    <comment ref="F99" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de inclusión. Es un artículo original de revista científica revisada por pares, aceptado en 2025 y publicado bajo copyright de 2026, con texto completo Open Access; estudia anomalías de tráfico vehicular en autopistas mediante Deep Learning y proporciona resultados cuantitativos de detección y localización.</t>
       </text>
     </comment>
-    <comment ref="F101" authorId="1" shapeId="0">
+    <comment ref="F101" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-3
 Motivo: Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
       </text>
     </comment>
-    <comment ref="F102" authorId="0" shapeId="0">
+    <comment ref="F102" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: el estudio cumple los criterios de inclusión por tratarse de un artículo original revisado por pares, publicado en 2026, con texto completo Open Access, contexto de tráfico vehicular urbano, arquitectura de Deep Learning y evaluación cuantitativa de detección de anomalías.</t>
       </text>
     </comment>
-    <comment ref="F103" authorId="0" shapeId="0">
+    <comment ref="F103" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de inclusión por ser un artículo científico original publicado en 2026, con texto completo Open Access, aplicación a anomalías visuales del tráfico vehicular, uso de redes neuronales profundas y evaluación cuantitativa.</t>
       </text>
     </comment>
-    <comment ref="F104" authorId="0" shapeId="0">
+    <comment ref="F104" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: el estudio cumple los criterios de inclusión. Es un artículo científico original de IEEE Transactions on Intelligent Vehicles, publicado en 2023, con texto completo accesible gratuitamente, datos reales de tráfico vehicular, arquitectura de Deep Learning y evaluación explícita de detección de anomalías.</t>
       </text>
     </comment>
-    <comment ref="F105" authorId="0" shapeId="0">
+    <comment ref="F105" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de inclusión por año (2024), publicación científica original, texto completo abierto, uso de Deep Learning y evaluación cuantitativa de accidentes de tráfico. Se incluye con advertencia de que UCF-Crime es un conjunto general de anomalías en videovigilancia y no exclusivamente de tráfico vehicular.</t>
@@ -4730,24 +4740,20 @@
           <t>cribado\pdf\R0029.pdf</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Excluir</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>CE-3</t>
-        </is>
-      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>No recuperado</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>three driving behaviors (normal, sleepy, and aggressive) on both highways and secondary roads (p. 3); "This section provides a comprehensive study of the proposed classification system for driving behavior." (p. 3)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>[Excluir CE-3] Estudio comparativo de clasificación de perfiles de conducción mediante ML, DL y ensamble PSO; no presenta una tarea específica de detección o anticipación de anomalías vehiculares.</t>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>[No recuperado] Sin texto completo de acceso abierto.</t>
         </is>
       </c>
     </row>
@@ -8592,7 +8598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8624,31 +8630,31 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>R0167</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>REHACER</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>Paradigma no identificable («aprendizaje federado»): elegir una opción de la lista con el PDF (https://jcbi.org/index.php/Main/article/download/1147/825). Si el PDF ya no se puede obtener, poner DECISIÓN TC = «No recuperado».</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>R0025</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Partición «No reportada» en la hoja 2 pero QA2 = 1 en la hoja 3: revisa uno de los dos.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>R0025</t>
+          <t>R0051</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -8663,14 +8669,14 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Partición «No reportada» en la hoja 2 pero QA2 = 1 en la hoja 3: revisa uno de los dos.</t>
+          <t>Partición aleatoria (411/35/148) pero QA2 = 1: según la escala sería 0.5.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>R0029</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -8685,14 +8691,14 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Se excluyó por CE-3 (clasifica perfiles normal/somnoliento/agresivo), pero R0032 (UAH-DriveSet, mismas tres clases), R0360, R0428 y R1029 se incluyeron. Decide con el mismo criterio para todos.</t>
+          <t>Caso límite: el DL extrae y reconstruye trayectorias y la anomalía se decide con reglas. Se mantiene incluido (regla de híbridos de CI-5); va al anexo de casos límite.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>R0051</t>
+          <t>R0986</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -8707,124 +8713,124 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Partición aleatoria (411/35/148) pero QA2 = 1: según la escala sería 0.5.</t>
+          <t>El texto analizado corresponde a Systems and Soft Computing (DOI 10.1016/j.sasc.2025.200254), pero el registro tiene DOI 10.1002/spy2.70136: confirma que el PDF es el del registro.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0024</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Revisar</t>
+          <t>Corregido «QA8 Limitaciones» → 0</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Caso límite: el DL extrae y reconstruye trayectorias y la anomalía se decide con reglas. Se mantiene incluido (regla de híbridos de CI-5); va al anexo de casos límite.</t>
+          <t>La hoja 2 dice «No reportadas»: la cita es trabajo futuro, no una limitación.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>R0986</t>
+          <t>R0024</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Revisar</t>
+          <t>Corregido «QA8 evidencia» → No reportado (solo trabajo futuro, p. 10)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>El texto analizado corresponde a Systems and Soft Computing (DOI 10.1016/j.sasc.2025.200254), pero el registro tiene DOI 10.1002/spy2.70136: confirma que el PDF es el del registro.</t>
+          <t>Coherente con la hoja 2.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>R0024</t>
+          <t>R0029</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA8 Limitaciones» → 0</t>
+          <t>Corregido «DECISIÓN TC» → No recuperado</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>La hoja 2 dice «No reportadas»: la cita es trabajo futuro, no una limitación.</t>
+          <t>El autor verificó que no hay texto completo en acceso abierto (la copia de SSRN no está disponible).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>R0024</t>
+          <t>R0029</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA8 evidencia» → No reportado (solo trabajo futuro, p. 10)</t>
+          <t>Corregido «CRITERIO» → None</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Coherente con la hoja 2.</t>
+          <t>No recuperado no lleva criterio.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>R0032</t>
+          <t>R0029</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Tipo de dato» → Multimodal</t>
+          <t>Corregido «Comentario» → [No recuperado] Sin texto completo de acceso abierto.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Acelerómetro, giroscopio y GPS del teléfono (UAH-DriveSet).</t>
+          <t>Coherente con las demás no recuperadas.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>R0052</t>
+          <t>R0032</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -8834,19 +8840,19 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «Tipo de dato» → Multimodal</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Intersecciones y rampas/puentes de carretera.</t>
+          <t>Acelerómetro, giroscopio y GPS del teléfono (UAH-DriveSet).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>R0080</t>
+          <t>R0052</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -8856,19 +8862,19 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Incidentes distintos en entrenamiento (23) y prueba (22).</t>
+          <t>Intersecciones y rampas/puentes de carretera.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>R0097</t>
+          <t>R0080</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -8878,19 +8884,19 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Ubicación y tipo de vía no reportados.</t>
+          <t>Incidentes distintos en entrenamiento (23) y prueba (22).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>R0119</t>
+          <t>R0097</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -8900,12 +8906,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Intersecciones y autopistas.</t>
+          <t>Ubicación y tipo de vía no reportados.</t>
         </is>
       </c>
     </row>
@@ -8922,19 +8928,19 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Partición estratificada sin separación temporal.</t>
+          <t>Intersecciones y autopistas.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>R0121</t>
+          <t>R0119</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -8944,19 +8950,19 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Urbano</t>
+          <t>Corregido «Partición» → Aleatoria</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Dos cruces peatonales de calle (35 mph) en Florida.</t>
+          <t>Partición estratificada sin separación temporal.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>R0167</t>
+          <t>R0121</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -8966,19 +8972,19 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → Urbano</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>«No se detallan particiones».</t>
+          <t>Dos cruces peatonales de calle (35 mph) en Florida.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>R0175</t>
+          <t>R0167</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -8988,19 +8994,19 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Paradigma» → No supervisado</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>No especifica el tipo de vía.</t>
+          <t>Releído el PDF: MGTGCN se entrena para predecir y reconstruir trayectorias (ADE/FDE, Tabla 1, p. 12), sin etiquetas de anomalía; las conductas anómalas se añaden después para evaluar: «adding a set of disruptive driving behaviors» (p. 12).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>R0185</t>
+          <t>R0167</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -9015,58 +9021,58 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>No describe la partición.</t>
+          <t>«No se detallan particiones».</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>R0190</t>
+          <t>R0175</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
+          <t>No especifica el tipo de vía.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
+          <t>No describe la partición.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0190</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -9076,12 +9082,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
+          <t>Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
         </is>
       </c>
     </row>
@@ -9098,12 +9104,12 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Cita del PDF.</t>
+          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
         </is>
       </c>
     </row>
@@ -9120,19 +9126,19 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Motivo.</t>
+          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>R0244</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -9142,19 +9148,19 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Incluir</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>«INCLUIDO» no es una opción de la lista.</t>
+          <t>Cita del PDF.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>R0249</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -9164,41 +9170,41 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>R0379</t>
+          <t>R0244</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Incluir</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Evalúa en una grabación highD no vista.</t>
+          <t>«INCLUIDO» no es una opción de la lista.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>R0389</t>
+          <t>R0249</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -9213,80 +9219,80 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
+          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0379</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA5 Código y datos» → 1</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
+          <t>Evalúa en una grabación highD no vista.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0389</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de DAD y CCD.</t>
+          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «QA5 Código y datos» → 1</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Vías urbanas e interurbanas.</t>
+          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -9301,36 +9307,36 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Conjunto externo ECVD solo para prueba.</t>
+          <t>Particiones oficiales de DAD y CCD.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>R0528</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
+          <t>Vías urbanas e interurbanas.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>R0537</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -9340,41 +9346,41 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Sin proporciones ni protocolo de separación.</t>
+          <t>Conjunto externo ECVD solo para prueba.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>R0596</t>
+          <t>R0528</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Partición insuficientemente reportada.</t>
+          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>R0598</t>
+          <t>R0537</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -9384,19 +9390,19 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Pista de pruebas; no es urbano ni autopista.</t>
+          <t>Sin proporciones ni protocolo de separación.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>R0601</t>
+          <t>R0596</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -9406,63 +9412,63 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de AI City Challenge.</t>
+          <t>Partición insuficientemente reportada.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0598</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
+          <t>Pista de pruebas; no es urbano ni autopista.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0601</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Conjunto de prueba de AI City Challenge.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>R0614</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -9472,63 +9478,63 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
+          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>R0658</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de los benchmarks.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>R0664</t>
+          <t>R0614</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Videos de prueba separados.</t>
+          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0658</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -9538,107 +9544,107 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>No detalla la partición.</t>
+          <t>Particiones oficiales de los benchmarks.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0664</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
+          <t>Videos de prueba separados.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>No detalla la partición.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>R0943</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
+          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>R1000</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>No indica qué escenas de NGSIM usa.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>R1010</t>
+          <t>R0943</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -9648,19 +9654,19 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Evaluado con autos de juguete en escenario controlado.</t>
+          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>R1013</t>
+          <t>R1000</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -9670,19 +9676,19 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba oficial de TADS.</t>
+          <t>No indica qué escenas de NGSIM usa.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R1010</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -9692,19 +9698,19 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Familia DL principal» → Otra</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>DeepWalk/Node2vec no es una GNN.</t>
+          <t>Evaluado con autos de juguete en escenario controlado.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>R1082</t>
+          <t>R1013</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -9719,14 +9725,14 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
+          <t>Conjunto de prueba oficial de TADS.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>R1092</t>
+          <t>R1014</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -9736,19 +9742,19 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «Familia DL principal» → Otra</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>División 80/20 de videos sin otro criterio.</t>
+          <t>DeepWalk/Node2vec no es una GNN.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>R1100</t>
+          <t>R1082</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -9758,19 +9764,19 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
+          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>R1138</t>
+          <t>R1092</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -9780,19 +9786,19 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Aleatoria</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>No desagrega urbano/autopista.</t>
+          <t>División 80/20 de videos sin otro criterio.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R1100</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -9802,19 +9808,19 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Objetos caídos sobre la calzada.</t>
+          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R1138</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -9824,41 +9830,41 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Solo dice que entrena y valida 100 épocas.</t>
+          <t>No desagrega urbano/autopista.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>R1166</t>
+          <t>R1148</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>Objetos caídos sobre la calzada.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>R1185</t>
+          <t>R1148</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -9868,54 +9874,98 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>No clasifica las imágenes por tipo de vía.</t>
+          <t>Solo dice que entrena y valida 100 épocas.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>R1202</t>
+          <t>R1166</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Separación por sesiones de conducción.</t>
+          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
+          <t>R1185</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>No clasifica las imágenes por tipo de vía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>R1202</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Separación por sesiones de conducción.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
           <t>R1214</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
         <is>
           <t>No informa proporciones ni criterio de división.</t>
         </is>
@@ -12062,118 +12112,122 @@
       <c r="X20" s="4" t="n"/>
     </row>
     <row r="21" ht="43.2" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>R0167</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>A Personalized Federated Learning Framework for Post-Event Forensic Traffic Analysis in Autonomous Vehicle Systems</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>cribado\pdf\R0167.pdf</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Trayectorias GPS</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Urbano</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>No especificado; se utilizan datos simulados CARLA y subconjuntos Comma.ai distribuidos en 3 clientes federados; no se reportan cantidades de vehículos, trayectorias, registros ni instancias de anomalías</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>Inyectadas/sintéticas</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Aprendizaje federado personalizado con entrenamiento local y agregación global; detección de anomalías mediante comportamientos anormales introducidos en los escenarios; no se especifica completamente el procedimiento de etiquetado ni el protocolo de partición</t>
         </is>
       </c>
-      <c r="J21" s="9" t="n"/>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>No supervisado</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>Grafos (GNN)</t>
         </is>
       </c>
-      <c r="L21" s="9" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>Personalized Lightweight Federated Learning (PLFL) con arquitectura MGTGCN; aprendizaje de trayectorias y detección de anomalías mediante fusión temporal y espacial; agregación federada personalizada según divergencia de modelos; Dynamic Model Pruning para reducir comunicación</t>
         </is>
       </c>
-      <c r="M21" s="9" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>Comportamiento de conducción</t>
         </is>
       </c>
-      <c r="O21" s="9" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>Precision, Recall y ROC-AUC para detección de anomalías; Average Displacement Error (ADE) y Final Displacement Error (FDE) para reconstrucción de trayectorias; tamaño de actualizaciones en MB para comunicación</t>
         </is>
       </c>
-      <c r="P21" s="9" t="inlineStr">
+      <c r="P21" s="5" t="inlineStr">
         <is>
           <t>Precision=89.3%, Recall=84.7%, ROC-AUC=0.921; PLFL ADE=1.98 m y FDE=4.55 m; FedAvg ADE=2.35 m y FDE=5.70 m; reducción de comunicación aproximada del 28%</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr">
         <is>
           <t>Datos simulados CARLA con comportamientos de conducción, colisiones y anomalías de ruta; subconjuntos reales Comma.ai; tres clientes: urbano, intersecciones y autopista/suburbano; tamaño exacto del conjunto de datos no especificado</t>
         </is>
       </c>
-      <c r="R21" s="9" t="inlineStr">
+      <c r="R21" s="5" t="inlineStr">
         <is>
           <t>Construcción de grafos espaciotemporales con nodos correspondientes a ubicaciones o segmentos viales y aristas de conectividad; extracción de características de telemetría; proyección a 64 dimensiones; fusión TCN-GCN-GAT; agregación personalizada; poda dinámica de parámetros de baja magnitud</t>
         </is>
       </c>
-      <c r="S21" s="9" t="inlineStr">
+      <c r="S21" s="7" t="inlineStr">
         <is>
           <t>No reportada</t>
         </is>
       </c>
-      <c r="T21" s="9" t="inlineStr">
+      <c r="T21" s="5" t="inlineStr">
         <is>
           <t>Centralized MGTGCN; Federated Learning FedAvg; Personalized FL/PLFL; comparación con y sin Dynamic Model Pruning; no se presenta tabla cuantitativa de Precision, Recall y ROC-AUC por cada baseline</t>
         </is>
       </c>
-      <c r="U21" s="9" t="inlineStr">
+      <c r="U21" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="V21" s="9" t="inlineStr">
+      <c r="V21" s="5" t="inlineStr">
         <is>
           <t>PLFL mejora ADE frente a FedAvg de 2.35 m a 1.98 m y FDE de 5.70 m a 4.55 m; alcanza Precision=89.3%, Recall=84.7% y ROC-AUC=0.921 en anomalías; reduce tamaño de actualización de 22.5 MB a 16.1 MB; mejora adaptación a distribuciones heterogéneas entre clientes</t>
         </is>
       </c>
-      <c r="W21" s="9" t="inlineStr">
+      <c r="W21" s="5" t="inlineStr">
         <is>
           <t>Enfoque forense posterior al evento sin evaluación en tiempo real; no se reportan tamaños exactos ni particiones de datasets; simulación CARLA con brecha respecto al mundo real; escasa representación de anomalías extremas; falta validación operacional a gran escala; no se evalúa resistencia a clientes maliciosos; inconsistencias entre tabla y figura de comunicación; no se proporciona código ni configuración experimental completa</t>
         </is>
       </c>
-      <c r="X21" s="9" t="inlineStr">
+      <c r="X21" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>

</xml_diff>

<commit_message>
Auditoría de coherencia: 5 exclusiones (R1014, R0666 CE-4; R0032, R0185 CE-3; R0072 CE-1) → 72 incluidos; hojas de re-cribado ciego TA (100) y TC (30)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxN9W1XmdV2QxsHjBBQujW
</commit_message>
<xml_diff>
--- a/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
+++ b/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
@@ -222,16 +222,70 @@
 Motivo: Coherente con las demás no recuperadas.</t>
       </text>
     </comment>
+    <comment ref="E6" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Incluir
+Motivo: Perfilado del conductor por viaje (igual que R0321, R0660 y R1046, CE-3).</t>
+      </text>
+    </comment>
     <comment ref="F6" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica: cumple los criterios de inclusión por ser un artículo original de conferencia ACM publicado en 2026, con texto completo disponible, aplicación a conducción vehicular real, modelos de Deep Learning y evaluación cuantitativa de comportamientos de riesgo. Se incluye como clasificación supervisada de conducción normal, agresiva y somnolienta, no como detección no supervisada de anomalías desconocidas.</t>
       </text>
     </comment>
+    <comment ref="G6" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Página 1: título, autores, conferencia ICIIT 2026, DOI y licencia CC BY 4.0. Página 3, sección 3.1: UAH-DriveSet, más de 500 minutos, seis conductores, carreteras y vías secundarias, tres comportamientos. Página 3, sección 3.2: partición estratificada 70% entrenamiento, 15% validación y 15% prueba. Página 4, Figura 1: flujo de preprocesamiento, modelos ML/DL y ensamble metaheurístico. Página 5, Tabla 1: comparación de nueve modelos, con accuracy de 0.9989 para PSO Ensemble, 0.9983 para Attention
+Motivo: Hoja 1 y 2 del autor.</t>
+      </text>
+    </comment>
+    <comment ref="H6" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se incluye porque analiza comportamientos de conducción potencialmente anómalos mediante sensores de teléfonos inteligentes y arquitecturas profundas de clasificación temporal. Compara CatBoost, XGBoost, KNN y ExtraTrees con CNN 1D, BiLSTM, TCN y Attention-LSTM, y propone un ensamble de modelos optimizado mediante Particle Swarm Optimization. El mejor modelo alcanza accuracy global de 99.89% y recall de 95% para la clase minoritaria de somnolencia. No detecta accidentes ocurridos ni eventos anóm
+Motivo: Motivo.</t>
+      </text>
+    </comment>
     <comment ref="F7" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 —</t>
+      </text>
+    </comment>
+    <comment ref="E12" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Incluir
+Motivo: Mismo modelo (MHGNN-CPLE), mismos autores y mismos datos que R0102; se conserva R0102 (Scientific Reports, versión más completa).</t>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: MHGNN-CPLE: detección estática Accuracy=0.980, F1=0.967, AUC=0.985 (p. 21, Tabla 5); detección dinámica de accidentes Accuracy=0.950, F1=0.945, AUC=0.970 (p. 22, Tabla 7); predicción dinámica de accidentes Accuracy=0.940, F1=0.935, AUC=0.965 (p. 23, Tabla 8); generalización METR-LA→PEMS-BAY Accuracy=0.945, F1=0.940 (p. 24, Tabla 9).
+Motivo: Hojas 1 y 2 del autor.</t>
+      </text>
+    </comment>
+    <comment ref="H12" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: [Incluir] Investigación original de 2025 sobre detección y predicción de anomalías vehiculares en autopistas mediante Deep Learning. Propone MHGNN-CPLE, integrando fusión multimodal, redes neuronales de grafos heterogéneos y optimización CPLE. Utiliza METR-LA y PEMS-BAY, con información de velocidad, flujo y densidad vehicular; también describe integración de imágenes y variables ambientales. Evalúa accidentes, congestión, tráfico normal y alteraciones meteorológicas. Compara con AGC-LSTM y Atte
+Motivo: Motivo.</t>
+      </text>
+    </comment>
+    <comment ref="E23" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Incluir
+Motivo: Clasifica niveles de riesgo de interacción, no eventos anómalos (igual que R0635, excluido por CE-3).</t>
+      </text>
+    </comment>
+    <comment ref="G23" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Seguimiento vehicular: Accuracy=83%, Precision=0.83, Recall=0.83, F1=0.83 (p. 6, Tabla 3). Cambio de carril: Accuracy=76%, Precision=0.75, Recall=0.76, F1=0.76 (p. 6, Tabla 4). Comparación: CNN=77%/67%, Bi-LSTM=80%/70%, GNN=61%/63% y CNN-LSTM-Attention=83%/76% de Accuracy en seguimiento/cambio de carril. Pruebas t pareadas y Wilcoxon con 10 ejecuciones independientes: p&lt;0.01 (p. 7). Evaluación de seguimiento con 3656 muestras de prueba (p. 7, Tabla 5). F1 de alto riesgo=0.87 en seguimiento y 0.7
+Motivo: Hoja 1 del autor.</t>
+      </text>
+    </comment>
+    <comment ref="H23" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: [Incluir] Investigación experimental original sobre identificación y predicción de estados anómalos de riesgo en conducción vehicular mediante Deep Learning. Propone CNN-LSTM-Attention con cuadrícula espacial 3×3 centrada en el vehículo, integración de Time-to-Collision (TTC) e Interaction Strength (IS), y clasificación dinámica de riesgo bajo, moderado y alto. Validación con trayectorias reales recolectadas en seis túneles de montaña de Chongqing, China. Obtiene Accuracy=83% en seguimiento vehi
+Motivo: Motivo.</t>
       </text>
     </comment>
     <comment ref="F24" authorId="0" shapeId="0">
@@ -504,10 +558,28 @@
 No aplica; cumple los criterios de inclusión por ser un artículo original de revista científica de 2025, con acceso abierto al texto completo, modelo basado en Deep Learning y evaluación cuantitativa de incidentes de tráfico vehicular.</t>
       </text>
     </comment>
+    <comment ref="E74" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Incluir
+Motivo: YOLOv5s/DeepSORT solo siguen vehículos; la anomalía se decide con umbrales manuales (igual que R0037, R0235 y R1213, excluidos por CE-4).</t>
+      </text>
+    </comment>
     <comment ref="F74" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica; artículo original de revista científica, publicado en 2024, con texto completo abierto y evaluación cuantitativa de comportamientos anómalos en autopistas mediante un sistema que incorpora redes profundas. La inclusión es condicionada a que el protocolo acepte Deep Learning para obtener y reconstruir trayectorias, aunque la decisión final de anomalía se base en reglas.</t>
+      </text>
+    </comment>
+    <comment ref="G74" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: El artículo presenta un sistema de vigilancia multicámara compuesto por YOLOv5s y DeepSORT para detección y seguimiento, una red de reidentificación vehicular con atributos y atención, y una BiLSTM para reconstruir trayectorias en zonas ciegas (secciones 3.1–3.3, pp. 5–11). La detección de anomalías utiliza reglas sobre dirección, velocidad, desplazamiento y pendiente de trayectoria, definidas en la Tabla 1 (p. 8) y sección 3.3.5 (pp. 10–11). Se evalúan conducción en sentido contrario, exceso de
+Motivo: Hoja 2 del autor.</t>
+      </text>
+    </comment>
+    <comment ref="H74" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: El estudio resulta pertinente para la revisión porque detecta anomalías de conducción vehicular en escenarios reales y utiliza Deep Learning como componente fundamental de la adquisición, asociación y reconstrucción de trayectorias. No obstante, la detección final se determina mediante umbrales manuales, por lo que sus resultados no demuestran el rendimiento de un clasificador profundo de anomalías. Las comparaciones con StRDAN, VAnet, PRND, SAVER y HPGN corresponden a reidentificación de vehícu
+Motivo: Motivo.</t>
       </text>
     </comment>
     <comment ref="F75" authorId="1" shapeId="0">
@@ -588,10 +660,28 @@
 No aplica — Estudio original publicado en Sensors en 2026, con revisión por pares y texto completo Open Access; desarrolla y evalúa cuantitativamente un modelo de Deep Learning para detectar accidentes y anomalías del tráfico vehicular mediante videos de vigilancia.</t>
       </text>
     </comment>
+    <comment ref="E87" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Incluir
+Motivo: DeepWalk/Node2vec no es Deep Learning; la anomalía la deciden SVDD y reglas.</t>
+      </text>
+    </comment>
     <comment ref="F87" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 No aplica — Artículo original de investigación publicado en revista científica, dentro del periodo 2020–2026, con texto completo Open Access; aborda explícitamente la detección de trayectorias anómalas y regiones de tráfico vehicular anormal mediante aprendizaje neuronal de representaciones de grafos.</t>
+      </text>
+    </comment>
+    <comment ref="G87" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Evidencia: Wang, Ye y Tang, Road traffic anomaly monitoring and warning based on DeepWalk algorithm, Transportation Safety and Environment, 2023, 5:tdac049, DOI 10.1093/tse/tdac049. La sección 2, p. 2, describe aproximadamente mil millones de puntos GPS correspondientes a 6083400 pedidos de taxis Didi en Chengdu durante noviembre de 2016. La sección 4.1, p. 6, informa una base procesada de aproximadamente 4160000 trayectorias, de las cuales 2 % son anómalas. La sección 3.2, pp. 4–5, describe Dee
+Motivo: Hoja 2 del autor.</t>
+      </text>
+    </comment>
+    <comment ref="H87" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se incluye por su pertinencia directa para la detección de anomalías en tráfico vehicular mediante Deep Learning. El modelo aprende representaciones de la red vial a partir de trayectorias GPS reales y las utiliza en un sistema de detección y alerta de anomalías regionales. La contribución principal es combinar DeepWalk/Node2vec con SVDD y Apriori para identificar trayectorias anómalas, localizar regiones afectadas y estimar su propagación. La evaluación utiliza datos reales de Chengdu y un comp
+Motivo: Motivo.</t>
       </text>
     </comment>
     <comment ref="F88" authorId="1" shapeId="0">
@@ -4778,20 +4868,24 @@
           <t>cribado\pdf\R0032.pdf</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Incluir</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Página 1: título, autores, conferencia ICIIT 2026, DOI y licencia CC BY 4.0. Página 3, sección 3.1: UAH-DriveSet, más de 500 minutos, seis conductores, carreteras y vías secundarias, tres comportamientos. Página 3, sección 3.2: partición estratificada 70% entrenamiento, 15% validación y 15% prueba. Página 4, Figura 1: flujo de preprocesamiento, modelos ML/DL y ensamble metaheurístico. Página 5, Tabla 1: comparación de nueve modelos, con accuracy de 0.9989 para PSO Ensemble, 0.9983 para Attention-LSTM y 0.9967 para TCN. Página 5, Figura 2: curvas ROC. Página 6: conclusiones y discusión del rendimiento.</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Se incluye porque analiza comportamientos de conducción potencialmente anómalos mediante sensores de teléfonos inteligentes y arquitecturas profundas de clasificación temporal. Compara CatBoost, XGBoost, KNN y ExtraTrees con CNN 1D, BiLSTM, TCN y Attention-LSTM, y propone un ensamble de modelos optimizado mediante Particle Swarm Optimization. El mejor modelo alcanza accuracy global de 99.89% y recall de 95% para la clase minoritaria de somnolencia. No detecta accidentes ocurridos ni eventos anómalos desconocidos: reconoce tres clases previamente definidas de estilo de conducción. Se identifican riesgos metodológicos importantes: solo seis conductores; agrupación de sus datos antes de la partición; ausencia de evaluación independiente por conductor; aplicación de SMOTE y preprocesamiento sin precisar su ajuste exclusivo sobre entrenamiento; resultados prácticamente perfectos en varios modelos; y falta de experimentos repetidos o validación externa. El propio artículo advierte posibles problemas de particionamiento en modelos temporales. Estos factores deben considerarse al interpretar la precisión y al comparar el estudio con métodos de detección de anomalías en tráfico vial.</t>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Excluir</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>CE-3</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>UAH-DriveSet, seis conductores, tres comportamientos (normal, somnoliento y agresivo); clasificación supervisada en una de las tres categorías (p. 3, secciones 3.1-3.2).</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] Compara ML, DL y un ensamble PSO para perfilar al conductor (normal/somnoliento/agresivo); no detecta eventos anómalos del tráfico.</t>
         </is>
       </c>
     </row>
@@ -5006,20 +5100,24 @@
           <t>cribado\pdf\R0072.pdf</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Incluir</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>MHGNN-CPLE: detección estática Accuracy=0.980, F1=0.967, AUC=0.985 (p. 21, Tabla 5); detección dinámica de accidentes Accuracy=0.950, F1=0.945, AUC=0.970 (p. 22, Tabla 7); predicción dinámica de accidentes Accuracy=0.940, F1=0.935, AUC=0.965 (p. 23, Tabla 8); generalización METR-LA→PEMS-BAY Accuracy=0.945, F1=0.940 (p. 24, Tabla 9).</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>[Incluir] Investigación original de 2025 sobre detección y predicción de anomalías vehiculares en autopistas mediante Deep Learning. Propone MHGNN-CPLE, integrando fusión multimodal, redes neuronales de grafos heterogéneos y optimización CPLE. Utiliza METR-LA y PEMS-BAY, con información de velocidad, flujo y densidad vehicular; también describe integración de imágenes y variables ambientales. Evalúa accidentes, congestión, tráfico normal y alteraciones meteorológicas. Compara con AGC-LSTM y AttentionDeepST; incluye pruebas de robustez, ablación y generalización entre conjuntos de datos. Limitaciones: documentación insuficiente sobre el origen de todas las modalidades, inconsistencias en la descripción de las particiones y falta de validación de despliegue en tiempo real.</t>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Excluir</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>CE-1</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Propone MHGNN-CPLE evaluado en METR-LA y PEMS-BAY con generalización METR-LA→PEMS-BAY (pp. 21-23, Tablas 5, 7 y 8); R0102 (Duan, Sun y Liu, 2025) presenta el mismo marco con las mismas bases.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-1] Publicación paralela de R0102 (Sun y Liu, 2025); se incluye R0102 para no contar dos veces el mismo modelo.</t>
         </is>
       </c>
     </row>
@@ -5412,20 +5510,24 @@
           <t>cribado\pdf\R0185.pdf</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Incluir</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Seguimiento vehicular: Accuracy=83%, Precision=0.83, Recall=0.83, F1=0.83 (p. 6, Tabla 3). Cambio de carril: Accuracy=76%, Precision=0.75, Recall=0.76, F1=0.76 (p. 6, Tabla 4). Comparación: CNN=77%/67%, Bi-LSTM=80%/70%, GNN=61%/63% y CNN-LSTM-Attention=83%/76% de Accuracy en seguimiento/cambio de carril. Pruebas t pareadas y Wilcoxon con 10 ejecuciones independientes: p&lt;0.01 (p. 7). Evaluación de seguimiento con 3656 muestras de prueba (p. 7, Tabla 5). F1 de alto riesgo=0.87 en seguimiento y 0.79 en cambio de carril (pp. 7-8, Tablas 5-6).</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>[Incluir] Investigación experimental original sobre identificación y predicción de estados anómalos de riesgo en conducción vehicular mediante Deep Learning. Propone CNN-LSTM-Attention con cuadrícula espacial 3×3 centrada en el vehículo, integración de Time-to-Collision (TTC) e Interaction Strength (IS), y clasificación dinámica de riesgo bajo, moderado y alto. Validación con trayectorias reales recolectadas en seis túneles de montaña de Chongqing, China. Obtiene Accuracy=83% en seguimiento vehicular y 76% en cambio de carril, superando CNN, Bi-LSTM y GNN. PDF completo disponible con licencia CC BY 4.0. Limitaciones: datos restringidos a túneles de Chongqing, partición de entrenamiento/prueba insuficientemente documentada, ausencia de evaluación externa y falta de disponibilidad pública explícita del dataset. Predice estados de riesgo, no accidentes observados.</t>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Excluir</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>CE-3</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Clasificación del riesgo de seguimiento y cambio de carril en niveles bajo, moderado y alto: Accuracy 83 % y 76 % (p. 6, Tablas 3 y 4).</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] CNN-LSTM-Attention estima el nivel de riesgo de las interacciones en túneles; no detecta ni anticipa eventos anómalos.</t>
         </is>
       </c>
     </row>
@@ -7378,20 +7480,24 @@
           <t>cribado\pdf\R0666.pdf</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>Incluir</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="n"/>
-      <c r="G74" s="4" t="inlineStr">
-        <is>
-          <t>El artículo presenta un sistema de vigilancia multicámara compuesto por YOLOv5s y DeepSORT para detección y seguimiento, una red de reidentificación vehicular con atributos y atención, y una BiLSTM para reconstruir trayectorias en zonas ciegas (secciones 3.1–3.3, pp. 5–11). La detección de anomalías utiliza reglas sobre dirección, velocidad, desplazamiento y pendiente de trayectoria, definidas en la Tabla 1 (p. 8) y sección 3.3.5 (pp. 10–11). Se evalúan conducción en sentido contrario, exceso de velocidad, velocidad baja, estacionamiento y cambios peligrosos de carril mediante conteos de aciertos, omisiones y falsas detecciones en las Tablas 3–7 (pp. 16–17). El conjunto de reidentificación incluye 100 vehículos registrados en la autopista de circunvalación de Xi’an (p. 14).</t>
-        </is>
-      </c>
-      <c r="H74" s="4" t="inlineStr">
-        <is>
-          <t>El estudio resulta pertinente para la revisión porque detecta anomalías de conducción vehicular en escenarios reales y utiliza Deep Learning como componente fundamental de la adquisición, asociación y reconstrucción de trayectorias. No obstante, la detección final se determina mediante umbrales manuales, por lo que sus resultados no demuestran el rendimiento de un clasificador profundo de anomalías. Las comparaciones con StRDAN, VAnet, PRND, SAVER y HPGN corresponden a reidentificación de vehículos y no a detección de comportamientos anómalos. La evaluación de anomalías presenta conteos cuantitativos, pero no un contraste directo con detectores alternativos ni validación independiente de las etiquetas. Se recomienda incluirlo como arquitectura híbrida de procesamiento profundo y decisión basada en reglas, señalando expresamente esta característica en la síntesis metodológica.</t>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Excluir</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>CE-4</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>Reglas explícitas: sentido contrario si Num/f ≥ 0,2; velocidad anómala si la media de 10 fotogramas supera n o baja de m; estacionamiento si la posición no cambia en cinco fotogramas (sección 3.3.5, pp. 10-11; Tabla 1, p. 8).</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-4] El DL detecta, sigue y reidentifica vehículos; los comportamientos peligrosos se deciden con umbrales manuales.</t>
         </is>
       </c>
     </row>
@@ -7880,20 +7986,24 @@
           <t>cribado\pdf\R1014.pdf</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>Incluir</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="n"/>
-      <c r="G87" s="4" t="inlineStr">
-        <is>
-          <t>Evidencia: Wang, Ye y Tang, Road traffic anomaly monitoring and warning based on DeepWalk algorithm, Transportation Safety and Environment, 2023, 5:tdac049, DOI 10.1093/tse/tdac049. La sección 2, p. 2, describe aproximadamente mil millones de puntos GPS correspondientes a 6083400 pedidos de taxis Didi en Chengdu durante noviembre de 2016. La sección 4.1, p. 6, informa una base procesada de aproximadamente 4160000 trayectorias, de las cuales 2 % son anómalas. La sección 3.2, pp. 4–5, describe DeepWalk con caminatas aleatorias y aprendizaje neuronal Skip-Gram, su extensión mediante Node2vec, la delimitación de regiones anómalas con SVDD y la predicción de propagación mediante Apriori. La Tabla 4, p. 7, reporta TAD 89,18 % y TAP 24,97 % frente al baseline SDA de 77,86 % y 22,25 %, respectivamente.</t>
-        </is>
-      </c>
-      <c r="H87" s="4" t="inlineStr">
-        <is>
-          <t>Se incluye por su pertinencia directa para la detección de anomalías en tráfico vehicular mediante Deep Learning. El modelo aprende representaciones de la red vial a partir de trayectorias GPS reales y las utiliza en un sistema de detección y alerta de anomalías regionales. La contribución principal es combinar DeepWalk/Node2vec con SVDD y Apriori para identificar trayectorias anómalas, localizar regiones afectadas y estimar su propagación. La evaluación utiliza datos reales de Chengdu y un comparador estadístico no profundo. Como limitaciones metodológicas para la revisión, la decisión final de región anómala se apoya en SVDD, la procedencia de las etiquetas no se documenta exhaustivamente, la partición entrenamiento/prueba no está suficientemente especificada y las métricas TAD/TAP presentan definiciones poco transparentes respecto de los indicadores estándar de clasificación. Se recomienda incluirlo, pero interpretar sus porcentajes como métricas propias del artículo y no como precision, recall o F1.</t>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>Excluir</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>CE-4</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>DeepWalk genera caminatas aleatorias y aprende embeddings con Skip-Gram; SVDD determina las regiones anómalas (sección 3, pp. 3-5); umbral de coincidencia de trayectorias anómalas 0,463 (sección 4.2, p. 6).</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-4] El detector es DeepWalk/Node2vec (embedding superficial, no DL) más SVDD, Apriori y umbrales.</t>
         </is>
       </c>
     </row>
@@ -8598,7 +8708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8676,7 +8786,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0986</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -8691,29 +8801,29 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Caso límite: el DL extrae y reconstruye trayectorias y la anomalía se decide con reglas. Se mantiene incluido (regla de híbridos de CI-5); va al anexo de casos límite.</t>
+          <t>El texto analizado corresponde a Systems and Soft Computing (DOI 10.1016/j.sasc.2025.200254), pero el registro tiene DOI 10.1002/spy2.70136: confirma que el PDF es el del registro.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>R0986</t>
+          <t>R0024</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Revisar</t>
+          <t>Corregido «QA8 Limitaciones» → 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>El texto analizado corresponde a Systems and Soft Computing (DOI 10.1016/j.sasc.2025.200254), pero el registro tiene DOI 10.1002/spy2.70136: confirma que el PDF es el del registro.</t>
+          <t>La hoja 2 dice «No reportadas»: la cita es trabajo futuro, no una limitación.</t>
         </is>
       </c>
     </row>
@@ -8730,34 +8840,34 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA8 Limitaciones» → 0</t>
+          <t>Corregido «QA8 evidencia» → No reportado (solo trabajo futuro, p. 10)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>La hoja 2 dice «No reportadas»: la cita es trabajo futuro, no una limitación.</t>
+          <t>Coherente con la hoja 2.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>R0024</t>
+          <t>R0029</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA8 evidencia» → No reportado (solo trabajo futuro, p. 10)</t>
+          <t>Corregido «DECISIÓN TC» → No recuperado</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Coherente con la hoja 2.</t>
+          <t>El autor verificó que no hay texto completo en acceso abierto (la copia de SSRN no está disponible).</t>
         </is>
       </c>
     </row>
@@ -8774,12 +8884,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → No recuperado</t>
+          <t>Corregido «CRITERIO» → None</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>El autor verificó que no hay texto completo en acceso abierto (la copia de SSRN no está disponible).</t>
+          <t>No recuperado no lleva criterio.</t>
         </is>
       </c>
     </row>
@@ -8796,34 +8906,34 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → None</t>
+          <t>Corregido «Comentario» → [No recuperado] Sin texto completo de acceso abierto.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>No recuperado no lleva criterio.</t>
+          <t>Coherente con las demás no recuperadas.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>R0029</t>
+          <t>R0032</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [No recuperado] Sin texto completo de acceso abierto.</t>
+          <t>Corregido «Tipo de dato» → Multimodal</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Coherente con las demás no recuperadas.</t>
+          <t>Acelerómetro, giroscopio y GPS del teléfono (UAH-DriveSet).</t>
         </is>
       </c>
     </row>
@@ -8835,90 +8945,90 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Tipo de dato» → Multimodal</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Acelerómetro, giroscopio y GPS del teléfono (UAH-DriveSet).</t>
+          <t>Perfilado del conductor por viaje (igual que R0321, R0660 y R1046, CE-3).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>R0052</t>
+          <t>R0032</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Intersecciones y rampas/puentes de carretera.</t>
+          <t>Clasifica estilos/perfiles de conducción, no anomalías del tráfico.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>R0080</t>
+          <t>R0032</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → UAH-DriveSet, seis conductores, tres comportamientos (normal, somnoliento y agresivo); clasificación supervisada en una de las tres categorías (p. 3, secciones 3.1-3.2).</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Incidentes distintos en entrenamiento (23) y prueba (22).</t>
+          <t>Hoja 1 y 2 del autor.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>R0097</t>
+          <t>R0032</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] Compara ML, DL y un ensamble PSO para perfilar al conductor (normal/somnoliento/agresivo); no detecta eventos anómalos del tráfico.</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Ubicación y tipo de vía no reportados.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>R0119</t>
+          <t>R0052</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -8933,102 +9043,102 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Intersecciones y autopistas.</t>
+          <t>Intersecciones y rampas/puentes de carretera.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>R0119</t>
+          <t>R0072</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Partición estratificada sin separación temporal.</t>
+          <t>Mismo modelo (MHGNN-CPLE), mismos autores y mismos datos que R0102; se conserva R0102 (Scientific Reports, versión más completa).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>R0121</t>
+          <t>R0072</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Urbano</t>
+          <t>Corregido «CRITERIO» → CE-1</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Dos cruces peatonales de calle (35 mph) en Florida.</t>
+          <t>Versión menos completa del mismo estudio.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>R0167</t>
+          <t>R0072</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Paradigma» → No supervisado</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → Propone MHGNN-CPLE evaluado en METR-LA y PEMS-BAY con generalización METR-LA→PEMS-BAY (pp. 21-23, Tablas 5, 7 y 8); R0102 (Duan, Sun y Liu, 2025) presenta el mismo marco con las mismas bases.</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Releído el PDF: MGTGCN se entrena para predecir y reconstruir trayectorias (ADE/FDE, Tabla 1, p. 12), sin etiquetas de anomalía; las conductas anómalas se añaden después para evaluar: «adding a set of disruptive driving behaviors» (p. 12).</t>
+          <t>Hojas 1 y 2 del autor.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>R0167</t>
+          <t>R0072</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Comentario» → [Excluir CE-1] Publicación paralela de R0102 (Sun y Liu, 2025); se incluye R0102 para no contar dos veces el mismo modelo.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>«No se detallan particiones».</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>R0175</t>
+          <t>R0080</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -9038,19 +9148,19 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>No especifica el tipo de vía.</t>
+          <t>Incidentes distintos en entrenamiento (23) y prueba (22).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>R0185</t>
+          <t>R0097</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -9060,151 +9170,151 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>No describe la partición.</t>
+          <t>Ubicación y tipo de vía no reportados.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>R0190</t>
+          <t>R0119</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
+          <t>Intersecciones y autopistas.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0119</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → Aleatoria</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
+          <t>Partición estratificada sin separación temporal.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0121</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Entorno» → Urbano</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
+          <t>Dos cruces peatonales de calle (35 mph) en Florida.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0167</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
+          <t>Corregido «Paradigma» → No supervisado</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Cita del PDF.</t>
+          <t>Releído el PDF: MGTGCN se entrena para predecir y reconstruir trayectorias (ADE/FDE, Tabla 1, p. 12), sin etiquetas de anomalía; las conductas anómalas se añaden después para evaluar: «adding a set of disruptive driving behaviors» (p. 12).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0167</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Motivo.</t>
+          <t>«No se detallan particiones».</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>R0244</t>
+          <t>R0175</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Incluir</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>«INCLUIDO» no es una opción de la lista.</t>
+          <t>No especifica el tipo de vía.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>R0249</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -9214,41 +9324,41 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>Clasifica niveles de riesgo de interacción, no eventos anómalos (igual que R0635, excluido por CE-3).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>R0379</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Evalúa en una grabación highD no vista.</t>
+          <t>Estimación de riesgo, sin detección de anomalías.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>R0389</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -9258,41 +9368,41 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → Clasificación del riesgo de seguimiento y cambio de carril en niveles bajo, moderado y alto: Accuracy 83 % y 76 % (p. 6, Tablas 3 y 4).</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
+          <t>Hoja 1 del autor.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA5 Código y datos» → 1</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] CNN-LSTM-Attention estima el nivel de riesgo de las interacciones en túneles; no detecta ni anticipa eventos anómalos.</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0185</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -9302,63 +9412,63 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de DAD y CCD.</t>
+          <t>No describe la partición.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0190</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Vías urbanas e interurbanas.</t>
+          <t>Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Conjunto externo ECVD solo para prueba.</t>
+          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>R0528</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -9373,124 +9483,124 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
+          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>R0537</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Sin proporciones ni protocolo de separación.</t>
+          <t>Cita del PDF.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>R0596</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Partición insuficientemente reportada.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>R0598</t>
+          <t>R0244</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «DECISIÓN TC» → Incluir</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Pista de pruebas; no es urbano ni autopista.</t>
+          <t>«INCLUIDO» no es una opción de la lista.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>R0601</t>
+          <t>R0249</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de AI City Challenge.</t>
+          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0379</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
+          <t>Evalúa en una grabación highD no vista.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0389</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -9500,41 +9610,41 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>R0614</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «QA5 Código y datos» → 1</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
+          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>R0658</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -9549,14 +9659,14 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de los benchmarks.</t>
+          <t>Particiones oficiales de DAD y CCD.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>R0664</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -9566,19 +9676,19 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Videos de prueba separados.</t>
+          <t>Vías urbanas e interurbanas.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -9588,19 +9698,19 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>No detalla la partición.</t>
+          <t>Conjunto externo ECVD solo para prueba.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0528</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -9610,41 +9720,41 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
+          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0537</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Sin proporciones ni protocolo de separación.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>R0943</t>
+          <t>R0596</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -9659,14 +9769,14 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
+          <t>Partición insuficientemente reportada.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>R1000</t>
+          <t>R0598</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -9681,14 +9791,14 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>No indica qué escenas de NGSIM usa.</t>
+          <t>Pista de pruebas; no es urbano ni autopista.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>R1010</t>
+          <t>R0601</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -9698,85 +9808,85 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Evaluado con autos de juguete en escenario controlado.</t>
+          <t>Conjunto de prueba de AI City Challenge.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>R1013</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba oficial de TADS.</t>
+          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Familia DL principal» → Otra</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>DeepWalk/Node2vec no es una GNN.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>R1082</t>
+          <t>R0614</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
+          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>R1092</t>
+          <t>R0658</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -9786,19 +9896,19 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>División 80/20 de videos sin otro criterio.</t>
+          <t>Particiones oficiales de los benchmarks.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>R1100</t>
+          <t>R0664</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -9808,85 +9918,85 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
+          <t>Videos de prueba separados.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>R1138</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>No desagrega urbano/autopista.</t>
+          <t>YOLOv5s/DeepSORT solo siguen vehículos; la anomalía se decide con umbrales manuales (igual que R0037, R0235 y R1213, excluidos por CE-4).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
+          <t>Corregido «CRITERIO» → CE-4</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Objetos caídos sobre la calzada.</t>
+          <t>La decisión de anomalía no la toma una red profunda.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → Reglas explícitas: sentido contrario si Num/f ≥ 0,2; velocidad anómala si la media de 10 fotogramas supera n o baja de m; estacionamiento si la posición no cambia en cinco fotogramas (sección 3.3.5, pp. 10-11; Tabla 1, p. 8).</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Solo dice que entrena y valida 100 épocas.</t>
+          <t>Hoja 2 del autor.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>R1166</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -9896,19 +10006,19 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Comentario» → [Excluir CE-4] El DL detecta, sigue y reidentifica vehículos; los comportamientos peligrosos se deciden con umbrales manuales.</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>R1185</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -9918,54 +10028,472 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>No clasifica las imágenes por tipo de vía.</t>
+          <t>No detalla la partición.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>R1202</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Separación por sesiones de conducción.</t>
+          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
+          <t>R0929</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «CRITERIO» → CE-2</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>R0943</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → No reportada</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>R1000</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>No indica qué escenas de NGSIM usa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>R1010</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Evaluado con autos de juguete en escenario controlado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>R1013</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Conjunto de prueba oficial de TADS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>DeepWalk/Node2vec no es Deep Learning; la anomalía la deciden SVDD y reglas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «CRITERIO» → CE-4</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Sin componente profunda entrenada que decida la anomalía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «EVIDENCIA (cita y página)» → DeepWalk genera caminatas aleatorias y aprende embeddings con Skip-Gram; SVDD determina las regiones anómalas (sección 3, pp. 3-5); umbral de coincidencia de trayectorias anómalas 0,463 (sección 4.2, p. 6).</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Hoja 2 del autor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Comentario» → [Excluir CE-4] El detector es DeepWalk/Node2vec (embedding superficial, no DL) más SVDD, Apriori y umbrales.</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Motivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Familia DL principal» → Otra</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>DeepWalk/Node2vec no es una GNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>R1082</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>R1092</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Aleatoria</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>División 80/20 de videos sin otro criterio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>R1100</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>R1138</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>No desagrega urbano/autopista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>R1148</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Objetos caídos sobre la calzada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>R1148</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → No reportada</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Solo dice que entrena y valida 100 épocas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>R1166</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «CRITERIO» → CI-6</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>R1185</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>No clasifica las imágenes por tipo de vía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>R1202</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Separación por sesiones de conducción.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
           <t>R1214</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D81" s="4" t="inlineStr">
         <is>
           <t>No informa proporciones ni criterio de división.</t>
         </is>

</xml_diff>

<commit_message>
Reescribe el manuscrito (v3) con el corpus definitivo de 72 estudios
- Nuevo título y texto completo: método con CI-2 de acceso abierto, cribado
  asistido por IA verificado, auditoría de coherencia, corpus solo de la
  búsqueda, calidad por niveles y análisis de sensibilidad.
- Resultados RQ1-RQ6 con las cifras generadas y ejemplos de datasets
  compartidos (CCD, PeMS, FT-AED).
- Tablas generadas partibles (xltabular); tabla de datasets con conjuntos
  públicos nombrados; macros de sensibilidad y de calidad baja.
- Corrige el autor citado en la exclusión de R0072 (Duan et al., 2025).
- Paquete de Overleaf apunta a RSL_v3.tex e incluye estudios.bib.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxN9W1XmdV2QxsHjBBQujW
</commit_message>
<xml_diff>
--- a/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
+++ b/RSL/cribado/revision/REVISION_TEXTO_COMPLETO.xlsx
@@ -266,7 +266,7 @@
     </comment>
     <comment ref="H12" authorId="0" shapeId="0">
       <text>
-        <t>Antes: [Incluir] Investigación original de 2025 sobre detección y predicción de anomalías vehiculares en autopistas mediante Deep Learning. Propone MHGNN-CPLE, integrando fusión multimodal, redes neuronales de grafos heterogéneos y optimización CPLE. Utiliza METR-LA y PEMS-BAY, con información de velocidad, flujo y densidad vehicular; también describe integración de imágenes y variables ambientales. Evalúa accidentes, congestión, tráfico normal y alteraciones meteorológicas. Compara con AGC-LSTM y Atte
+        <t>Antes: [Excluir CE-1] Publicación paralela de R0102 (Sun y Liu, 2025); se incluye R0102 para no contar dos veces el mismo modelo.
 Motivo: Motivo.</t>
       </text>
     </comment>
@@ -294,6 +294,12 @@
 Motivo: Es tráfico vehicular (no CE-2): solo pronostica el flujo con MAE, no detecta anomalías.</t>
       </text>
     </comment>
+    <comment ref="H24" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: [Excluir - CE-2] El artículo aborda predicción de flujo vehicular mediante Deep LSTM y Mixture Deep LSTM utilizando datos simulados de tráfico y meteorología. Aunque incorpora escenarios posteriores a accidentes y condiciones de tráfico no habituales, los accidentes se consideran condiciones conocidas para pronosticar el flujo posterior, no eventos que el modelo deba detectar o clasificar. La variable de salida es el flujo vehicular previsto y la evaluación principal utiliza MAE. No se desarroll
+Motivo: Coherente con CE-3.</t>
+      </text>
+    </comment>
     <comment ref="E25" authorId="0" shapeId="0">
       <text>
         <t>Antes: Incluir
@@ -330,6 +336,12 @@
 Motivo: Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
       </text>
     </comment>
+    <comment ref="H31" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: [Excluir] Estudio original de 2020 sobre tráfico vehicular que utiliza un Variational Autoencoder (VAE) con datos reales de California (EE. UU.) e Inglaterra (Reino Unido). Aunque incluye una aplicación exploratoria a la detección de anomalías, no presenta evaluación cuantitativa específica de detección, como precisión, recall, F1 o AUROC, ni validación con etiquetas de anomalías. Las métricas numéricas principales evalúan predicción e imputación. Incumple CI-6; se registra CE-3 como motivo prin
+Motivo: Coherente con CI-6.</t>
+      </text>
+    </comment>
     <comment ref="F32" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
@@ -390,6 +402,12 @@
 Motivo: Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
       </text>
     </comment>
+    <comment ref="H42" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se excluye de la síntesis principal de estudios de detección de anomalías vehiculares mediante Deep Learning por ausencia de evaluación cuantitativa específica del detector. Raiyn (2022) propone Computational Data Science para analizar datos de velocidad, posición GNSS y calidad de datos obtenidos mediante teléfonos inteligentes, sensores y dispositivos Ublox. Considera anomalías asociadas a accidentes, congestión, ruido, interferencia y pérdida de información. Define condiciones anormales media
+Motivo: Comentario conciso para el anexo.</t>
+      </text>
+    </comment>
     <comment ref="F43" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
@@ -432,6 +450,12 @@
 Motivo: Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
       </text>
     </comment>
+    <comment ref="H51" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se excluye por CE-3 porque, aunque desarrolla un método de Deep Learning directamente relacionado con la detección de accidentes vehiculares, no aporta resultados cuantitativos verificables y comparables de detección de anomalías. Las curvas de entrenamiento y los gráficos de puntuaciones de anomalía no equivalen a una evaluación de clasificación frente a etiquetas de referencia. Tampoco se documentan claramente el tamaño final del conjunto de prueba, el número de accidentes evaluados, los falso
+Motivo: Coherente con CI-6.</t>
+      </text>
+    </comment>
     <comment ref="F52" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
@@ -466,6 +490,12 @@
       <text>
         <t>Texto original:
 CE-5: Tipo de publicación no elegible; tesis de maestría, sin evidencia de publicación de este documento como artículo revisado por pares.</t>
+      </text>
+    </comment>
+    <comment ref="H57" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se excluye exclusivamente por CE-5, dado que el texto completo disponible es una tesis de maestría y el protocolo exige estudios originales publicados en revistas o congresos con revisión por pares. El estudio sí satisface los requisitos temáticos, temporales y metodológicos: aborda detección de incidentes vehiculares, utiliza una arquitectura profunda TabNet entrenada de forma supervisada y proporciona métricas cuantitativas de detección. Sus resultados proceden de incidentes simulados, no de u
+Motivo: Comentario conciso para el anexo.</t>
       </text>
     </comment>
     <comment ref="F59" authorId="1" shapeId="0">
@@ -504,12 +534,24 @@
 No aplica</t>
       </text>
     </comment>
+    <comment ref="H63" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se incluye por abordar detección explícita de comportamientos de conducción peligrosos en transporte vehicular terrestre mediante un modelo Deep Learning entrenado y evaluado cuantitativamente. La detección de fatiga y distracción del conductor se considera una subcategoría de anomalías de comportamiento vehicular. Es necesario diferenciar estos resultados de la detección de accidentes o anomalías de flujo de tráfico, que el estudio no evalúa cuantitativamente. Presenta limitaciones de reproduci
+Motivo: Comentario conciso para el anexo.</t>
+      </text>
+    </comment>
     <comment ref="F64" authorId="0" shapeId="0">
       <text>
         <t>Antes: CE-4
 Motivo: Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
       </text>
     </comment>
+    <comment ref="H64" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se excluye del corpus principal de la revisión sistemática porque no cumple el requisito metodológico obligatorio de emplear un modelo Deep Learning para detectar anomalías del tráfico vehicular. La contribución consiste en comparar clasificadores convencionales y métodos de boosting basados en árboles para estimar la severidad de accidentes conocidos, utilizando atributos meteorológicos, temporales y contextuales. LightGBM alcanza ROC-AUC de 0.866 en la Tabla 3, pero este resultado evalúa clasi
+Motivo: Coherente con CE-3.</t>
+      </text>
+    </comment>
     <comment ref="F65" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
@@ -522,18 +564,36 @@
 CE-5: documento disponible como prepublicación arXiv, sin evidencia de publicación arbitrada en revista o congreso dentro del PDF. El manuscrito se identifica como arXiv:2505.02613v1, fechado el 5 de mayo de 2025, y no presenta DOI editorial, nombre de congreso, revista ni datos de aceptación. La exclusión se refiere al estado de publicación verificable de esta versión; no implica que el trabajo carezca de calidad científica ni descarta una eventual versión publicada posteriormente.</t>
       </text>
     </comment>
+    <comment ref="H66" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Excluir por CE-5 conforme al requisito de incluir exclusivamente investigaciones originales publicadas en revistas o congresos con revisión por pares. El contenido técnico sí corresponde al tema de la revisión: detección de anomalías reales en tráfico vehicular mediante Deep Learning, con evaluación cuantitativa y etiquetas verificadas por expertos. La exclusión no se debe a falta de pertinencia temática, ausencia de aprendizaje profundo ni indisponibilidad del texto completo. Se conserva la ext
+Motivo: Comentario conciso para el anexo.</t>
+      </text>
+    </comment>
     <comment ref="F67" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-5: prepublicación arXiv sin acreditación de revisión por pares en la versión PDF examinada. El documento figura como arXiv:2303.05000v1 [cs.LG], fechado el 9 de marzo de 2023, sin nombre de revista, congreso, volumen, páginas editoriales ni DOI de publicación. La decisión corresponde exclusivamente a esta versión documental y deberá reconsiderarse si se identifica una publicación arbitrada equivalente.</t>
       </text>
     </comment>
+    <comment ref="H67" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Excluir por CE-5 de acuerdo con el protocolo de la revisión sistemática, que exige estudios originales publicados en revistas o congresos revisados por pares. El manuscrito aborda directamente la detección de trayectorias anómalas de vehículos mediante Deep Learning y aporta experimentos comparativos en dos datasets públicos. Es importante registrar que las anomalías son ataques adversariales generados artificialmente, no accidentes, congestiones o conductas anómalas reales anotadas por expertos
+Motivo: Comentario conciso para el anexo.</t>
+      </text>
+    </comment>
     <comment ref="F69" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
 CE-3: El estudio se centra en predicción de riesgo de colisión y no demuestra un sistema de detección explícita de anomalías vehiculares en tráfico general. Aunque clasifica muestras peligrosas y presenta métricas de clasificación, los escenarios peligrosos se preseleccionan mediante TTC &lt; 3 s; el propio artículo reconoce que todavía es necesario identificar esos periodos en aplicaciones reales.</t>
       </text>
     </comment>
+    <comment ref="H69" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Excluir por CE-3. Li et al. (2026) presentan LLMG + ST, una arquitectura híbrida de GPT-2-LoRA, GAT y LSTM para predecir riesgo de colisión en seguimiento vehicular a partir de trayectorias highD. Aunque la investigación es original, utiliza Deep Learning y obtiene resultados cuantitativos, no evalúa la detección autónoma de anomalías sobre tráfico no preseleccionado. Sus 240 eventos de riesgo se identifican previamente mediante un criterio TTC &lt; 3 s, y el modelo pronostica la peligrosidad de ve
+Motivo: Comentario conciso para el anexo.</t>
+      </text>
+    </comment>
     <comment ref="F70" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
@@ -544,6 +604,12 @@
       <text>
         <t>Texto original:
 CE-3: el estudio no evalúa cuantitativamente la detección de anomalías en tráfico vehicular. Aunque propone un modelo Deep Learning para analizar conducción peligrosa, su tarea experimental es la predicción de series temporales y del nivel macroscópico de riesgo generado mediante reglas difusas, sin contrastar decisiones de anomalía contra etiquetas de referencia independientes.</t>
+      </text>
+    </comment>
+    <comment ref="H71" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se excluye Li, Lin y Chou (2022), DOI 10.1109/ACCESS.2022.3171247, por CE-3. El artículo es pertinente al análisis de conducción peligrosa y emplea una red recurrente profunda fuzzy-macro LSTM con datos reales de diez conductores, pero su evaluación se concentra en pronosticar variables vehiculares y una puntuación agregada de riesgo calculada mediante un sistema de inferencia difusa. El mejor modelo obtiene MAE 0,613, RMSE 0,733 y MSE 0,521 para la predicción del nivel de riesgo, resultados que
+Motivo: Comentario conciso para el anexo.</t>
       </text>
     </comment>
     <comment ref="F72" authorId="1" shapeId="0">
@@ -618,6 +684,12 @@
 No aplica; estudio original publicado en una conferencia ACM de 2024, con texto completo disponible. Desarrolla y evalúa una CNN para reconocer una conducta anómala de conducción, específicamente el uso del teléfono móvil, y la integra en un sistema de seguridad vehicular.</t>
       </text>
     </comment>
+    <comment ref="H79" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se incluye exclusivamente por la detección supervisada mediante CNN de una conducta vehicular anómala observable en imágenes del conductor: uso del teléfono durante la conducción. No debe clasificarse como estudio que demuestra detección de accidentes mediante Deep Learning, porque el módulo de accidentes depende del acelerómetro y no se presenta una evaluación independiente de accidentes con CNN. La matriz de confusión contiene únicamente 32 imágenes y no se documenta la independencia entre suj
+Motivo: Comentario conciso para el anexo.</t>
+      </text>
+    </comment>
     <comment ref="F80" authorId="1" shapeId="0">
       <text>
         <t>Texto original:
@@ -640,6 +712,12 @@
       <text>
         <t>Texto original:
 CE-3 — El estudio no desarrolla ni evalúa cuantitativamente un método de detección de anomalías en tráfico vehicular. Su objetivo principal es la predicción no lineal del flujo de tráfico mediante una red LSTM de dos capas y una infraestructura IoT. Aunque menciona incidentes, condiciones anormales, valores atípicos y fallos de sensores, no presenta etiquetas de anomalías viales, una regla de clasificación de eventos anómalos ni métricas específicas de detección.</t>
+      </text>
+    </comment>
+    <comment ref="H83" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Excluir por CE-3. Aunque el artículo cumple los criterios de año, publicación científica, acceso al texto completo, contexto vehicular y uso de Deep Learning, no satisface el criterio central de la revisión: detección explícita y cuantitativamente evaluada de anomalías del tráfico vehicular. La LSTM predice conteos y velocidades, y los resultados MSE, MAE, RMSE y R² miden error de pronóstico, no capacidad para detectar accidentes, congestión atípica o comportamientos anómalos. El filtrado de out
+Motivo: Comentario conciso para el anexo.</t>
       </text>
     </comment>
     <comment ref="F84" authorId="1" shapeId="0">
@@ -754,6 +832,12 @@
       <text>
         <t>Antes: CE-3
 Motivo: Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+      </text>
+    </comment>
+    <comment ref="H101" authorId="0" shapeId="0">
+      <text>
+        <t>Antes: Se excluye durante la revisión de texto completo porque la contribución principal es el diseño e implementación de una plataforma de videovigilancia vehicular con detección, seguimiento, calibración y análisis de trayectorias. El uso de Deep Learning está documentado, y la Figura 9 demuestra que el sistema contempla incidentes viales, pero no existe un experimento reproducible que cuantifique su capacidad para distinguir incidentes reales de situaciones normales. No se informa tamaño del conjunt
+Motivo: Coherente con CI-6.</t>
       </text>
     </comment>
     <comment ref="F102" authorId="1" shapeId="0">
@@ -5117,7 +5201,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>[Excluir CE-1] Publicación paralela de R0102 (Sun y Liu, 2025); se incluye R0102 para no contar dos veces el mismo modelo.</t>
+          <t>[Excluir CE-1] Publicación paralela de R0102 (Duan et al., 2025); se incluye R0102 para no contar dos veces el mismo modelo.</t>
         </is>
       </c>
     </row>
@@ -5567,9 +5651,9 @@
           <t>El estudio propone Deep LSTM y Mixture Deep LSTM para pronóstico del flujo vehicular en horas punta y escenarios posteriores a accidentes (p. 3, sección 3.1). Utiliza datos simulados inspirados en tráfico y meteorología de Los Ángeles (p. 3, sección 3.2). Reporta MAE=4 vehículos/minuto en horas punta y MAE=6 vehículos/minuto durante los primeros 30 minutos posteriores a accidentes (p. 4, secciones 4.3-4.4). La Figura 2 (p. 5) compara SimpleCNN=76.99%, CNN_LSTM=60% y BERT_CNN/FullIntegration=46.5%, pero estas métricas no corresponden a una evaluación explícita de detección de anomalías. No presenta etiquetas de anomalía, detección de incidentes ni métricas específicas de identificación de eventos anómalos.</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>[Excluir - CE-2] El artículo aborda predicción de flujo vehicular mediante Deep LSTM y Mixture Deep LSTM utilizando datos simulados de tráfico y meteorología. Aunque incorpora escenarios posteriores a accidentes y condiciones de tráfico no habituales, los accidentes se consideran condiciones conocidas para pronosticar el flujo posterior, no eventos que el modelo deba detectar o clasificar. La variable de salida es el flujo vehicular previsto y la evaluación principal utiliza MAE. No se desarrolla ni valida un método específico de detección de anomalías en tráfico vehicular. Se excluye por falta de correspondencia con el objetivo central de la revisión sistemática, no por ausencia de Deep Learning ni de texto completo.</t>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] Pronostica el flujo con Deep LSTM y Mixture Deep LSTM (MAE) en horas punta y tras accidentes; los accidentes son una condición de entrada, no eventos que se detecten.</t>
         </is>
       </c>
     </row>
@@ -5841,9 +5925,9 @@
           <t>Sección 7.2, pp. 13–16: exploración de anomalías mediante el espacio latente del VAE; p. 15: la metodología de detección automática y su precisión se dejan como trabajo futuro.</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>[Excluir] Estudio original de 2020 sobre tráfico vehicular que utiliza un Variational Autoencoder (VAE) con datos reales de California (EE. UU.) e Inglaterra (Reino Unido). Aunque incluye una aplicación exploratoria a la detección de anomalías, no presenta evaluación cuantitativa específica de detección, como precisión, recall, F1 o AUROC, ni validación con etiquetas de anomalías. Las métricas numéricas principales evalúan predicción e imputación. Incumple CI-6; se registra CE-3 como motivo principal.</t>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CI-6] VAE para imputación, reducción de dimensión y pronóstico; la detección de anomalías es exploratoria (espacio latente) y no se evalúa con etiquetas ni métricas de detección.</t>
         </is>
       </c>
     </row>
@@ -6259,9 +6343,9 @@
           <t>Página 1: resumen y DOI; declara detección de anomalías y uso de Deep Learning. Página 4, Figuras 1–3: comparación de velocidades y variaciones estadísticas ante condiciones anormales. Página 5, sección 3.2: umbral ilustrativo de reducción de velocidad de 30 km/h y pruebas de diferencias entre estaciones. Página 9, sección 4.11: red descrita genéricamente mediante entrada, capas ocultas y salida. Página 10, Figura 7: flujo CDS para detección, identificación de fuente y localización. Página 13, Figura 10: esquema genérico de neuronas, pesos y activación. Página 15, Tabla 4: estadísticas de regresión para condiciones con y sin ruido, no métricas de clasificación. Página 15, Figuras 13–14: visualización de anomalías de posicionamiento y comparación gráfica CDS frente a ML sin indicadores cuantitativos de detección. Página 16, conclusiones: se afirma una mejora de pronóstico, pero no se cuantifica la detección de anomalías.</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>Se excluye de la síntesis principal de estudios de detección de anomalías vehiculares mediante Deep Learning por ausencia de evaluación cuantitativa específica del detector. Raiyn (2022) propone Computational Data Science para analizar datos de velocidad, posición GNSS y calidad de datos obtenidos mediante teléfonos inteligentes, sensores y dispositivos Ublox. Considera anomalías asociadas a accidentes, congestión, ruido, interferencia y pérdida de información. Define condiciones anormales mediante desviaciones de velocidad y diferencias espaciales y temporales; presenta una red neuronal conceptual y un procedimiento de entrenamiento y prueba. Sin embargo, no identifica con precisión el conjunto experimental, las etiquetas de referencia, la arquitectura profunda, el tamaño de entrenamiento y prueba ni los parámetros de aprendizaje. La Tabla 4 informa Multiple R, R², R² ajustado, desviación estándar y asimetría en presencia y ausencia de ruido, pero esos valores no son métricas de detección. Las Figuras 13 y 14 muestran resultados visuales sin tasas de aciertos o errores. Por tanto, no es posible extraer un rendimiento comparable con los estudios incluidos. Se conserva como antecedente conceptual sobre anomalías de velocidad, calidad de datos y posicionamiento vehicular, sin incorporarlo al análisis cuantitativo principal.</t>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CI-6] Propone un enfoque de ciencia de datos con DL para anomalías de velocidad, pero no reporta métricas de detección (precision, recall, F1 o AUC) ni etiquetas de referencia.</t>
         </is>
       </c>
     </row>
@@ -6597,9 +6681,9 @@
           <t>Artículo de conferencia publicado en Electronic Imaging 2023, DOI 10.2352/EI.2023.35.3.MOBMU-364, con texto completo accesible de 12 páginas. Propone un sistema de detección de accidentes vehiculares que integra eliminación de fondo mediante U²-Net, detección y seguimiento de objetos mediante YOLO-R y DeepSORT, y redes generativas adversarias para identificar anomalías en escenas de vigilancia. Compara variantes GAN sin conexiones de salto, GAN con conexiones de salto y GAN con conexiones de salto y atención (secciones Methodology y Results, pp. 3-8). Utiliza imágenes procedentes de videos de vigilancia y describe conjuntos públicos de referencia como UCFCrime, Street Scene y ShanghaiTech (Tabla 1, p. 5). Las Figuras 10 y 13 (pp. 10-11) muestran señales de distancia de Mahalanobis y error adversarial, mientras que las Figuras 11 y 12 (p. 10) presentan curvas de entrenamiento. No se proporciona una tabla de resultados de detección con precision, recall, F1-score, AUC, tasa de falsos positivos o matriz de confusión, ni un protocolo cuantitativo suficientemente documentado que permita verificar el desempeño sobre accidentes etiquetados.</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>Se excluye por CE-3 porque, aunque desarrolla un método de Deep Learning directamente relacionado con la detección de accidentes vehiculares, no aporta resultados cuantitativos verificables y comparables de detección de anomalías. Las curvas de entrenamiento y los gráficos de puntuaciones de anomalía no equivalen a una evaluación de clasificación frente a etiquetas de referencia. Tampoco se documentan claramente el tamaño final del conjunto de prueba, el número de accidentes evaluados, los falsos positivos y negativos ni una comparación numérica completa entre las variantes propuestas. No se excluye por CE-2 ni CE-4, puesto que el dominio es tráfico vehicular y sí se utilizan redes profundas. El estudio puede citarse como antecedente metodológico, pero no debe incorporarse a la síntesis cuantitativa principal bajo los criterios establecidos.</t>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CI-6] YOLO-R, DeepSORT y GAN para detectar accidentes en video, sin tabla de resultados de detección (precision, recall, F1 o AUC) frente a accidentes etiquetados.</t>
         </is>
       </c>
     </row>
@@ -6829,9 +6913,9 @@
           <t>La portada identifica explícitamente el documento como "A Thesis Presented in Partial Fulfillment of the Requirements for the Degree Master of Science", presentada en Arizona State University y aprobada en mayo de 2024 (PDF, p. 1). El documento tiene estructura de tesis, con capítulos de introducción, trabajos relacionados, metodología, experimentos, resultados y conclusión, y no presenta datos editoriales que acrediten su publicación como artículo de revista o congreso revisado por pares. En cuanto al contenido científico, propone IncidentNet, basado en tres modelos TabNet para detección, localización y estimación de gravedad de incidentes de tráfico mediante sensores dispersos. Emplea datos microscópicos generados con SUMO y calibrados con conteos vehiculares reales de Tempe, Arizona. Reporta en el escenario urbano DR de 98 %, FAR de 6,26 %, MTTD de 197,44 segundos y F1 de 92,70 % (Tabla 5.1, PDF p. 25). También presenta resultados en autopistas, con DR de 99 %, FAR de 4,17 % y MTTD de 70 segundos (Tabla 5.2, PDF p. 28).</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>Se excluye exclusivamente por CE-5, dado que el texto completo disponible es una tesis de maestría y el protocolo exige estudios originales publicados en revistas o congresos con revisión por pares. El estudio sí satisface los requisitos temáticos, temporales y metodológicos: aborda detección de incidentes vehiculares, utiliza una arquitectura profunda TabNet entrenada de forma supervisada y proporciona métricas cuantitativas de detección. Sus resultados proceden de incidentes simulados, no de una validación operacional con accidentes reales, lo que constituye una limitación adicional, pero no el motivo principal de exclusión. Se recomienda conservar este registro como literatura relacionada y comprobar por separado si existe un artículo revisado por pares derivado de la tesis, evitando incluir automáticamente la tesis como si fuera dicho artículo.</t>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-5] El texto completo disponible es una tesis de maestría; no se encontró una versión revisada por pares de acceso abierto.</t>
         </is>
       </c>
     </row>
@@ -7057,9 +7141,9 @@
           <t>Artículo original de conferencia publicado en ACM CMNM 2026 (pp. 284–290), con texto completo disponible bajo licencia Creative Commons Attribution 4.0. Desarrolla un sistema de asistencia para la seguridad de camiones que integra un modelo YOLOv8n entrenado para reconocer comportamientos peligrosos del conductor, incluyendo bostezos, uso del teléfono y tabaquismo, así como estados de apertura y cierre de ojos. En la sección 3 (p. 289) se informa un conjunto propio de 6000 imágenes etiquetadas, dividido en entrenamiento y prueba con proporción 10:1 y utilizado para entrenar el modelo durante 120 épocas. La Tabla 1 (p. 286) presenta el mAP@0.5 de seis clases y la Tabla 2 (p. 289) proporciona precisión, recall, mAP@0.5 y mAP@0.5:0.95 para cuatro comportamientos. El mAP@0.5 global declarado es 95.8 %.</t>
         </is>
       </c>
-      <c r="H63" s="4" t="inlineStr">
-        <is>
-          <t>Se incluye por abordar detección explícita de comportamientos de conducción peligrosos en transporte vehicular terrestre mediante un modelo Deep Learning entrenado y evaluado cuantitativamente. La detección de fatiga y distracción del conductor se considera una subcategoría de anomalías de comportamiento vehicular. Es necesario diferenciar estos resultados de la detección de accidentes o anomalías de flujo de tráfico, que el estudio no evalúa cuantitativamente. Presenta limitaciones de reproducibilidad, ausencia de modelos comparativos y escasa documentación del dataset y de la generalización.</t>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-2] YOLOv8n reconoce fatiga, bostezos, uso del teléfono y tabaquismo del conductor de camión en imágenes de cabina: es monitoreo del conductor.</t>
         </is>
       </c>
     </row>
@@ -7099,9 +7183,9 @@
           <t>Artículo original publicado en AICCC 2023 (ACM, pp. 179–188), con texto completo disponible. La sección 4, Proposed Solution (p. 183), establece que la propuesta utiliza exclusivamente Random Forest, XGBoost y LightGBM para clasificación multiclase de la gravedad de accidentes. La sección 4.1 (p. 183) describe el Countrywide Traffic Accident Dataset, con aproximadamente 2.8 millones de accidentes estadounidenses entre febrero de 2016 y diciembre de 2021. La sección 5 y la Tabla 3 (pp. 186–187) presentan resultados únicamente de esos tres algoritmos. Las referencias a CNN, GAN y otras redes profundas en las secciones 3.1–3.3 y Tabla 1 (pp. 181–185) corresponden a antecedentes bibliográficos y no a experimentos propios.</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr">
-        <is>
-          <t>Se excluye del corpus principal de la revisión sistemática porque no cumple el requisito metodológico obligatorio de emplear un modelo Deep Learning para detectar anomalías del tráfico vehicular. La contribución consiste en comparar clasificadores convencionales y métodos de boosting basados en árboles para estimar la severidad de accidentes conocidos, utilizando atributos meteorológicos, temporales y contextuales. LightGBM alcanza ROC-AUC de 0.866 en la Tabla 3, pero este resultado evalúa clasificación de severidad y no detección de accidentes. El estudio puede servir como antecedente contextual sobre predicción de severidad y tratamiento del desbalance de clases, sin incorporarse a la síntesis de modelos profundos de detección de anomalías.</t>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] Clasifica la gravedad de accidentes ya registrados (Random Forest, XGBoost, LightGBM); no detecta incidentes y tampoco usa DL.</t>
         </is>
       </c>
     </row>
@@ -7179,9 +7263,9 @@
           <t>El trabajo presenta un sistema de detección de anomalías de tráfico por carril en autopistas de Indiana, Estados Unidos, mediante datos extraídos de cámaras de vigilancia. Emplea YOLOv5x-CBAM y Deep SORT para detectar y seguir vehículos; genera series temporales de conteo, ocupación y porcentaje de camiones; utiliza un VQ-VAE sobre espectrogramas de transformada wavelet continua, reglas de congestión e Isolation Forest. El conjunto procede de 8746 videos de 15 minutos captados por cinco cámaras durante seis meses; se reportan 46 clips anómalos validados por expertos, 73139 muestras normales por carril y 341 muestras anómalas etiquetadas (sección III, pp. 2–4). La Tabla III (p. 6) reporta para el sistema completo accuracy 0,9787, precisión 0,8431, recall 1,0 y F1 0,9149. La Tabla II presenta comparaciones con Isolation Forest, OWAM, TimeVQVAE-AD y TranAD. La portada identifica el documento como arXiv:2505.02613v1, sin indicar publicación revisada por pares.</t>
         </is>
       </c>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>Excluir por CE-5 conforme al requisito de incluir exclusivamente investigaciones originales publicadas en revistas o congresos con revisión por pares. El contenido técnico sí corresponde al tema de la revisión: detección de anomalías reales en tráfico vehicular mediante Deep Learning, con evaluación cuantitativa y etiquetas verificadas por expertos. La exclusión no se debe a falta de pertinencia temática, ausencia de aprendizaje profundo ni indisponibilidad del texto completo. Se conserva la extracción metodológica porque el estudio aporta un conjunto de datos de autopistas con resolución por carril y un sistema modular VQ-VAE, reglas e Isolation Forest. Si se identifica posteriormente una versión arbitrada del mismo trabajo, debe verificarse su equivalencia y reevaluarse el registro sin duplicarlo en Parsifal.</t>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-5] Preprint de arXiv (2505.02613) sin versión revisada por pares verificable.</t>
         </is>
       </c>
     </row>
@@ -7221,9 +7305,9 @@
           <t>El estudio propone dos métodos de detección de trayectorias vehiculares anómalas: aprendizaje contrastivo supervisado y reconstrucción no supervisada mediante un adversarial autoencoder con espacio latente semántico. Ambos utilizan un extractor profundo que combina convoluciones unidimensionales para trayectorias y redes neuronales de grafos para mapas e interacciones entre agentes (sección III, pp. 3–5; Figuras 2–3, pp. 4–5). Se evalúan sobre Argoverse 1 y Argoverse 2, con anomalías adversariales sintéticas de tipo aleatorio y direccional lateral generadas mediante perturbaciones de trayectorias históricas (secciones II.A y IV.A, pp. 2 y 5). Las Tablas I–IV (p. 6) reportan F1, ROC-AUC y PR-AUC; el mejor resultado supervisado es F1 0,99, ROC-AUC 0,98 y PR-AUC 0,99 en anomalías laterales de Argoverse 2. La pertinencia temática y la evaluación cuantitativa están acreditadas, pero no la publicación arbitrada.</t>
         </is>
       </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>Excluir por CE-5 de acuerdo con el protocolo de la revisión sistemática, que exige estudios originales publicados en revistas o congresos revisados por pares. El manuscrito aborda directamente la detección de trayectorias anómalas de vehículos mediante Deep Learning y aporta experimentos comparativos en dos datasets públicos. Es importante registrar que las anomalías son ataques adversariales generados artificialmente, no accidentes, congestiones o conductas anómalas reales anotadas por expertos. La exclusión se fundamenta en el estado editorial de la versión suministrada, no en falta de relevancia, ausencia de DL o falta de texto completo. Si se localiza una versión revisada por pares, deberá comprobarse su identidad bibliográfica y reevaluarse este mismo registro sin duplicarlo en Parsifal.</t>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-5] Preprint de arXiv (2303.05000) sin versión revisada por pares verificable.</t>
         </is>
       </c>
     </row>
@@ -7297,9 +7381,9 @@
           <t>Evidencia: sección 3.1, página 3, Figura 1: el flujo comienza con la selección de eventos peligrosos del conjunto highD mediante TTC &lt; 3 s y termina en predicción de riesgo. Sección 4.1, página 6: se identifican 240 eventos peligrosos y se indica expresamente que el caso verifica el método sobre eventos de alto riesgo predefinidos. Sección 4.3.1, página 6: las primeras 70 tramas sirven para predecir riesgo en las 30 posteriores. Tabla 3, página 10: Accuracy 0.956, F1 0.872 y AUC 0.985 corresponden a predicción/clasificación de riesgo. Conclusiones, página 11: los autores reconocen que el método aún no identifica automáticamente periodos peligrosos en conducción real.</t>
         </is>
       </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>Excluir por CE-3. Li et al. (2026) presentan LLMG + ST, una arquitectura híbrida de GPT-2-LoRA, GAT y LSTM para predecir riesgo de colisión en seguimiento vehicular a partir de trayectorias highD. Aunque la investigación es original, utiliza Deep Learning y obtiene resultados cuantitativos, no evalúa la detección autónoma de anomalías sobre tráfico no preseleccionado. Sus 240 eventos de riesgo se identifican previamente mediante un criterio TTC &lt; 3 s, y el modelo pronostica la peligrosidad de ventanas futuras. Los autores reconocen explícitamente que la aplicación real requerirá identificar primero los periodos peligrosos e incorporar datos de conducción segura. Se conserva como antecedente metodológico relacionado, pero no cumple el objetivo específico de detección de anomalías de esta revisión.</t>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] GPT-2-LoRA, GAT y LSTM predicen el riesgo de colisión en eventos peligrosos preseleccionados (TTC &lt; 3 s) de highD; no detecta anomalías sobre tráfico no preseleccionado.</t>
         </is>
       </c>
     </row>
@@ -7377,9 +7461,9 @@
           <t>Evidencia del PDF: sección II.A, página 47882, define la salida como grado macroscópico de conducción riesgosa calculado a partir de aceleraciones bruscas, frenadas bruscas y velocidad media por 100 km. Sección II.C y Tabla 1, páginas 47883–47884, presentan 27 reglas difusas para asignar riesgo bajo, medio o alto. Sección III.A, página 47886, describe datos reales OBD-II de diez participantes durante nueve meses. Sección III.B, página 47887, establece exclusivamente MAE, MSE y RMSE como métricas experimentales. Tablas 2 y 3, página 47888, y Tabla 4, página 47891, comparan errores de predicción frente a cinco redes neuronales. Figuras 22–24, página 47892, comparan valores reales y pronosticados de velocidad, frenadas y aceleraciones; no presentan evaluación de identificación de eventos anómalos.</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>Se excluye Li, Lin y Chou (2022), DOI 10.1109/ACCESS.2022.3171247, por CE-3. El artículo es pertinente al análisis de conducción peligrosa y emplea una red recurrente profunda fuzzy-macro LSTM con datos reales de diez conductores, pero su evaluación se concentra en pronosticar variables vehiculares y una puntuación agregada de riesgo calculada mediante un sistema de inferencia difusa. El mejor modelo obtiene MAE 0,613, RMSE 0,733 y MSE 0,521 para la predicción del nivel de riesgo, resultados que no constituyen métricas de detección de anomalías. No se informa validación de eventos peligrosos detectados mediante etiquetas independientes, ni métricas de clasificación normal/anómalo, sensibilidad, precisión, F1 o AUC. La existencia de reglas de riesgo alto no basta para demostrar capacidad de detección. El artículo puede conservarse como referencia contextual sobre predicción del riesgo de conducción, pero no debe incorporarse a la síntesis cuantitativa de detección de anomalías.</t>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] LSTM difusa que pronostica variables de conducción y un nivel de riesgo calculado con reglas difusas; solo reporta MAE, MSE y RMSE.</t>
         </is>
       </c>
     </row>
@@ -7689,9 +7773,9 @@
           <t>La sección 3.4, pp. 279–280, describe una CNN personalizada entrenada con imágenes etiquetadas como phone_holding y not_holding. Se declara un conjunto de 11745 imágenes procedentes de How drive 3d driver distraction y fotografías propias, sección 3.4.1, p. 279. La Figura 2, p. 280, presenta tres capas convolucionales seguidas de capas densas. La Figura 7, p. 282, presenta una matriz de confusión de 32 imágenes: TN=9, FP=0, FN=0 y TP=23, equivalente a exactitud, precisión, sensibilidad y F1 del 100 % en esa muestra. La sección 4.1, p. 280, informa exactitud de entrenamiento del 100 %. La detección de accidentes se realiza mediante el acelerómetro ADXL335, mientras que velocidad y alcohol se supervisan mediante GPS y sensor MQ3, secciones 3.3 y 4.3, pp. 278 y 282. La Tabla 3, p. 286, declara 90 % de detección y reducción de accidentes, sin presentar denominadores, matriz de confusión ni protocolo de evaluación que respalden ese porcentaje.</t>
         </is>
       </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>Se incluye exclusivamente por la detección supervisada mediante CNN de una conducta vehicular anómala observable en imágenes del conductor: uso del teléfono durante la conducción. No debe clasificarse como estudio que demuestra detección de accidentes mediante Deep Learning, porque el módulo de accidentes depende del acelerómetro y no se presenta una evaluación independiente de accidentes con CNN. La matriz de confusión contiene únicamente 32 imágenes y no se documenta la independencia entre sujetos o sesiones de entrenamiento y prueba. Tampoco se presentan comparaciones cuantitativas entre modelos profundos bajo el mismo conjunto de prueba, intervalos de confianza ni evidencia de generalización externa. El 90 % de la Tabla 3 no debe utilizarse como métrica validada de detección de anomalías por Deep Learning. Es pertinente para la revisión en la subcategoría de comportamiento de conducción, con calidad experimental limitada.</t>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-2] La CNN clasifica si el conductor sostiene el teléfono en imágenes de cabina; el módulo de accidentes depende del acelerómetro y no se evalúa con DL.</t>
         </is>
       </c>
     </row>
@@ -7845,9 +7929,9 @@
           <t>El artículo es una investigación original publicada en 2025 en Systems and Soft Computing, volumen 7, artículo 200254, DOI 10.1016/j.sasc.2025.200254, con texto completo Open Access. La sección 3.2, p. 3, describe aproximadamente 9,1 millones de observaciones recogidas entre enero y junio de 2024 mediante 35 sensores IoT en 12 intersecciones y 23 segmentos de autopista. La sección 3.3, pp. 3–5, presenta una arquitectura LSTM de dos capas con 64 y 32 unidades, destinada a predecir variables del tráfico. La Tabla 6, p. 6, informa MSE de prueba 0,0953, MAE 0,0728, R² 0,8976 y RMSE 0,3087. La Tabla 7, p. 7, compara errores de predicción con media móvil, regresión lineal, Auto ARIMA y LSTM de una capa. La sección 4.3, p. 10, menciona adaptación a incidentes y bloqueos inesperados, pero únicamente como estudios de caso de predicción, sin matriz de confusión ni métricas de detección de anomalías. La sección 4.2, p. 10, informa 99,9 % de detección de condiciones anómalas del sistema de monitoreo en 30 segundos; este resultado corresponde a supervisión operativa de la infraestructura, no a la detección de anomalías vehiculares mediante la LSTM.</t>
         </is>
       </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>Excluir por CE-3. Aunque el artículo cumple los criterios de año, publicación científica, acceso al texto completo, contexto vehicular y uso de Deep Learning, no satisface el criterio central de la revisión: detección explícita y cuantitativamente evaluada de anomalías del tráfico vehicular. La LSTM predice conteos y velocidades, y los resultados MSE, MAE, RMSE y R² miden error de pronóstico, no capacidad para detectar accidentes, congestión atípica o comportamientos anómalos. El filtrado de outliers mediante IQR es una operación estadística de limpieza de datos y no constituye el método profundo de detección. Las alertas por incertidumbre, los fallos de sensores y las condiciones anómalas del sistema tampoco demuestran detección vial. No corresponde CE-4 porque sí emplea LSTM; tampoco CE-6 porque el PDF completo está disponible. Registrar CE-3 como motivo principal de exclusión en Parsifal.</t>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CE-3] LSTM con IoT para pronosticar el flujo de autopista; menciona eventos anormales, pero no los etiqueta ni evalúa su detección.</t>
         </is>
       </c>
     </row>
@@ -8529,9 +8613,9 @@
           <t>Página 1, resumen: se describe un sistema de procesamiento de video, compresión de redes neuronales, detección nocturna, seguimiento de vehículos y análisis de comportamiento; se afirma que funciona en distintas localidades de China, pero sin cifras de desempeño. Página 2, Figura 1: arquitectura modular de vigilancia. Página 4, Figuras 5 y 6: ejemplos visuales de detección y seguimiento de vehículos. Página 5, sección 5.2 y Figura 9: demostración de un incidente de circulación en sentido contrario, sin comparación con etiquetas de referencia ni resultados cuantitativos. Página 5, conclusión: se reiteran beneficios operativos y despliegue parcial en Zhejiang, sin métricas de anomalías.</t>
         </is>
       </c>
-      <c r="H101" s="4" t="inlineStr">
-        <is>
-          <t>Se excluye durante la revisión de texto completo porque la contribución principal es el diseño e implementación de una plataforma de videovigilancia vehicular con detección, seguimiento, calibración y análisis de trayectorias. El uso de Deep Learning está documentado, y la Figura 9 demuestra que el sistema contempla incidentes viales, pero no existe un experimento reproducible que cuantifique su capacidad para distinguir incidentes reales de situaciones normales. No se informa tamaño del conjunto de prueba, número de incidentes, falsos positivos, falsos negativos, precision, recall, F1, AUROC ni tiempo de detección. El estudio puede citarse como antecedente de arquitectura de sistemas de vigilancia, pero no debe incorporarse a la síntesis de efectividad de métodos de detección de anomalías. Criterio principal: CE-3; no corresponde excluirlo por ausencia de Deep Learning.</t>
+      <c r="H101" s="7" t="inlineStr">
+        <is>
+          <t>[Excluir CI-6] Plataforma de videovigilancia con detección y seguimiento de vehículos; muestra ejemplos de incidentes, pero no reporta métricas de detección.</t>
         </is>
       </c>
     </row>
@@ -8708,7 +8792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9126,7 +9210,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [Excluir CE-1] Publicación paralela de R0102 (Sun y Liu, 2025); se incluye R0102 para no contar dos veces el mismo modelo.</t>
+          <t>Corregido «Comentario» → [Excluir CE-1] Publicación paralela de R0102 (Duan et al., 2025); se incluye R0102 para no contar dos veces el mismo modelo.</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -9446,7 +9530,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>R0192</t>
+          <t>R0190</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -9456,12 +9540,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] Pronostica el flujo con Deep LSTM y Mixture Deep LSTM (MAE) en horas punta y tras accidentes; los accidentes son una condición de entrada, no eventos que se detecten.</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
+          <t>Coherente con CE-3.</t>
         </is>
       </c>
     </row>
@@ -9478,12 +9562,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
+          <t>Releído el PDF: la detección solo se valida de forma visual (face validation); la única métrica cuantitativa (RMSE, Tabla 1) es de imputación.</t>
         </is>
       </c>
     </row>
@@ -9500,12 +9584,12 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Cita del PDF.</t>
+          <t>Sin evaluación cuantitativa de la detección (igual que R0249 y R0389).</t>
         </is>
       </c>
     </row>
@@ -9522,19 +9606,19 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → "we employ a face validation approach. In this approach, we visually examine the pace time series of various zones" (p. 10, sección IV-E); "Table 1 presents the mean and standard deviation of RMSE across 10 trials of inference-phase imputation" (p. 9, sección IV-C).</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Motivo.</t>
+          <t>Cita del PDF.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>R0244</t>
+          <t>R0192</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -9544,19 +9628,19 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Incluir</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] SI-DMSeq (encoder-decoder LSTM con atención, Manhattan, huracán Sandy y tormenta de 2010) detecta disrupciones con una carta de control sobre el error de reconstrucción, pero no las evalúa contra etiquetas: no hay precision, recall, F1, AUC ni tasa de detección; la única métrica numérica (RMSE) es de imputación.</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>«INCLUIDO» no es una opción de la lista.</t>
+          <t>Motivo.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>R0249</t>
+          <t>R0244</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -9566,41 +9650,41 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «DECISIÓN TC» → Incluir</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>«INCLUIDO» no es una opción de la lista.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>R0379</t>
+          <t>R0249</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Evalúa en una grabación highD no vista.</t>
+          <t>Sí trata la detección de anomalías, pero solo de forma exploratoria y sin métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>R0389</t>
+          <t>R0249</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -9610,129 +9694,129 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] VAE para imputación, reducción de dimensión y pronóstico; la detección de anomalías es exploratoria (espacio latente) y no se evalúa con etiquetas ni métricas de detección.</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
+          <t>Coherente con CI-6.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0379</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Corregido «QA5 Código y datos» → 1</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
+          <t>Evalúa en una grabación highD no vista.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>R0403</t>
+          <t>R0389</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de DAD y CCD.</t>
+          <t>Trata anomalías de tráfico pero no reporta métricas de detección: es CI-6 (igual que R0249, R0528 y R1166).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0389</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → Ambos</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] Propone un enfoque de ciencia de datos con DL para anomalías de velocidad, pero no reporta métricas de detección (precision, recall, F1 o AUC) ni etiquetas de referencia.</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Vías urbanas e interurbanas.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>R0501</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «QA5 Código y datos» → 1</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Conjunto externo ECVD solo para prueba.</t>
+          <t>Código con DOI (ETS) y datasets públicos (DAD, CCD, A3D): ambos públicos.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>R0528</t>
+          <t>R0403</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
+          <t>Particiones oficiales de DAD y CCD.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>R0537</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -9742,19 +9826,19 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → Ambos</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Sin proporciones ni protocolo de separación.</t>
+          <t>Vías urbanas e interurbanas.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>R0596</t>
+          <t>R0501</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -9764,85 +9848,85 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Partición insuficientemente reportada.</t>
+          <t>Conjunto externo ECVD solo para prueba.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>R0598</t>
+          <t>R0528</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «CRITERIO» → CI-6</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Pista de pruebas; no es urbano ni autopista.</t>
+          <t>Detecta accidentes con DL, pero no reporta métricas de detección: es CI-6, no CE-3.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>R0601</t>
+          <t>R0528</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Comentario» → [Excluir CI-6] YOLO-R, DeepSORT y GAN para detectar accidentes en video, sin tabla de resultados de detección (precision, recall, F1 o AUC) frente a accidentes etiquetados.</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de AI City Challenge.</t>
+          <t>Coherente con CI-6.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0537</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
+          <t>Sin proporciones ni protocolo de separación.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>R0604</t>
+          <t>R0585</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -9852,41 +9936,41 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Comentario» → [Excluir CE-5] El texto completo disponible es una tesis de maestría; no se encontró una versión revisada por pares de acceso abierto.</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>R0614</t>
+          <t>R0596</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-3</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
+          <t>Partición insuficientemente reportada.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>R0658</t>
+          <t>R0598</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -9896,19 +9980,19 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Particiones oficiales de los benchmarks.</t>
+          <t>Pista de pruebas; no es urbano ni autopista.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>R0664</t>
+          <t>R0601</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -9923,14 +10007,14 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Videos de prueba separados.</t>
+          <t>Conjunto de prueba de AI City Challenge.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -9945,14 +10029,14 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>YOLOv5s/DeepSORT solo siguen vehículos; la anomalía se decide con umbrales manuales (igual que R0037, R0235 y R1213, excluidos por CE-4).</t>
+          <t>Monitoreo del conductor dentro de la cabina (fatiga, bostezos, teléfono): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -9962,19 +10046,19 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-4</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>La decisión de anomalía no la toma una red profunda.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0604</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -9984,19 +10068,19 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Corregido «EVIDENCIA (cita y página)» → Reglas explícitas: sentido contrario si Num/f ≥ 0,2; velocidad anómala si la media de 10 fotogramas supera n o baja de m; estacionamiento si la posición no cambia en cinco fotogramas (sección 3.3.5, pp. 10-11; Tabla 1, p. 8).</t>
+          <t>Corregido «Comentario» → [Excluir CE-2] YOLOv8n reconoce fatiga, bostezos, uso del teléfono y tabaquismo del conductor de camión en imágenes de cabina: es monitoreo del conductor.</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Hoja 2 del autor.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0614</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -10006,41 +10090,41 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [Excluir CE-4] El DL detecta, sigue y reidentifica vehículos; los comportamientos peligrosos se deciden con umbrales manuales.</t>
+          <t>Corregido «CRITERIO» → CE-3</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Motivo.</t>
+          <t>Predice la gravedad de accidentes ya registrados; CE-3 va antes que CE-4 en el orden fijo.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>R0666</t>
+          <t>R0614</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] Clasifica la gravedad de accidentes ya registrados (Random Forest, XGBoost, LightGBM); no detecta incidentes y tampoco usa DL.</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>No detalla la partición.</t>
+          <t>Coherente con CE-3.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0618</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -10050,19 +10134,19 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Corregido «DECISIÓN TC» → Excluir</t>
+          <t>Corregido «Comentario» → [Excluir CE-5] Preprint de arXiv (2505.02613) sin versión revisada por pares verificable.</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>R0929</t>
+          <t>R0622</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -10072,63 +10156,63 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CE-2</t>
+          <t>Corregido «Comentario» → [Excluir CE-5] Preprint de arXiv (2303.05000) sin versión revisada por pares verificable.</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo del conductor dentro de la cabina.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>R0943</t>
+          <t>R0635</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] GPT-2-LoRA, GAT y LSTM predicen el riesgo de colisión en eventos peligrosos preseleccionados (TTC &lt; 3 s) de highD; no detecta anomalías sobre tráfico no preseleccionado.</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>R1000</t>
+          <t>R0646</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] LSTM difusa que pronostica variables de conducción y un nivel de riesgo calculado con reglas difusas; solo reporta MAE, MSE y RMSE.</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>No indica qué escenas de NGSIM usa.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>R1010</t>
+          <t>R0658</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -10138,19 +10222,19 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Evaluado con autos de juguete en escenario controlado.</t>
+          <t>Particiones oficiales de los benchmarks.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>R1013</t>
+          <t>R0664</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -10165,14 +10249,14 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba oficial de TADS.</t>
+          <t>Videos de prueba separados.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -10187,14 +10271,14 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>DeepWalk/Node2vec no es Deep Learning; la anomalía la deciden SVDD y reglas.</t>
+          <t>YOLOv5s/DeepSORT solo siguen vehículos; la anomalía se decide con umbrales manuales (igual que R0037, R0235 y R1213, excluidos por CE-4).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -10209,14 +10293,14 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Sin componente profunda entrenada que decida la anomalía.</t>
+          <t>La decisión de anomalía no la toma una red profunda.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -10226,7 +10310,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Corregido «EVIDENCIA (cita y página)» → DeepWalk genera caminatas aleatorias y aprende embeddings con Skip-Gram; SVDD determina las regiones anómalas (sección 3, pp. 3-5); umbral de coincidencia de trayectorias anómalas 0,463 (sección 4.2, p. 6).</t>
+          <t>Corregido «EVIDENCIA (cita y página)» → Reglas explícitas: sentido contrario si Num/f ≥ 0,2; velocidad anómala si la media de 10 fotogramas supera n o baja de m; estacionamiento si la posición no cambia en cinco fotogramas (sección 3.3.5, pp. 10-11; Tabla 1, p. 8).</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -10238,7 +10322,7 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -10248,7 +10332,7 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Comentario» → [Excluir CE-4] El detector es DeepWalk/Node2vec (embedding superficial, no DL) más SVDD, Apriori y umbrales.</t>
+          <t>Corregido «Comentario» → [Excluir CE-4] El DL detecta, sigue y reidentifica vehículos; los comportamientos peligrosos se deciden con umbrales manuales.</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -10260,7 +10344,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>R1014</t>
+          <t>R0666</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -10270,85 +10354,85 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Familia DL principal» → Otra</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>DeepWalk/Node2vec no es una GNN.</t>
+          <t>No detalla la partición.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>R1082</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
+          <t>La CNN solo reconoce si el conductor sostiene el teléfono (imagen de cabina): CE-2 lo excluye expresamente.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>R1092</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Aleatoria</t>
+          <t>Corregido «CRITERIO» → CE-2</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>División 80/20 de videos sin otro criterio.</t>
+          <t>Monitoreo del conductor dentro de la cabina.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>R1100</t>
+          <t>R0929</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Comentario» → [Excluir CE-2] La CNN clasifica si el conductor sostiene el teléfono en imágenes de cabina; el módulo de accidentes depende del acelerómetro y no se evalúa con DL.</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>R1138</t>
+          <t>R0943</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -10358,41 +10442,41 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>No desagrega urbano/autopista.</t>
+          <t>Sin procedimiento de selección ni conjunto de prueba.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R0986</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
+          <t>Corregido «Comentario» → [Excluir CE-3] LSTM con IoT para pronosticar el flujo de autopista; menciona eventos anormales, pero no los etiqueta ni evalúa su detección.</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Objetos caídos sobre la calzada.</t>
+          <t>Comentario conciso para el anexo.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>R1148</t>
+          <t>R1000</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -10402,41 +10486,41 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → No reportada</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Solo dice que entrena y valida 100 épocas.</t>
+          <t>No indica qué escenas de NGSIM usa.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>R1166</t>
+          <t>R1010</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Corregido «CRITERIO» → CI-6</t>
+          <t>Corregido «Entorno» → No reportado</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+          <t>Evaluado con autos de juguete en escenario controlado.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>R1185</t>
+          <t>R1013</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -10446,54 +10530,362 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Entorno» → No reportado</t>
+          <t>Corregido «Partición» → Prueba independiente</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>No clasifica las imágenes por tipo de vía.</t>
+          <t>Conjunto de prueba oficial de TADS.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>R1202</t>
+          <t>R1014</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Corregido «Partición» → Prueba independiente</t>
+          <t>Corregido «DECISIÓN TC» → Excluir</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Separación por sesiones de conducción.</t>
+          <t>DeepWalk/Node2vec no es Deep Learning; la anomalía la deciden SVDD y reglas.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «CRITERIO» → CE-4</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Sin componente profunda entrenada que decida la anomalía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «EVIDENCIA (cita y página)» → DeepWalk genera caminatas aleatorias y aprende embeddings con Skip-Gram; SVDD determina las regiones anómalas (sección 3, pp. 3-5); umbral de coincidencia de trayectorias anómalas 0,463 (sección 4.2, p. 6).</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Hoja 2 del autor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Comentario» → [Excluir CE-4] El detector es DeepWalk/Node2vec (embedding superficial, no DL) más SVDD, Apriori y umbrales.</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Motivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>R1014</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Familia DL principal» → Otra</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>DeepWalk/Node2vec no es una GNN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>R1082</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Conjunto de prueba de MAAD (con ajuste de hiperparámetros en parte de él).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>R1092</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Aleatoria</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>División 80/20 de videos sin otro criterio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>R1100</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>DoTA/CCD sin clasificación por tipo de vía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>R1138</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>No desagrega urbano/autopista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>R1148</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Categoría de anomalía» → Evento/otro</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Objetos caídos sobre la calzada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>R1148</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → No reportada</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Solo dice que entrena y valida 100 épocas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>R1166</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «CRITERIO» → CI-6</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Es un sistema de detección de incidentes sin métricas de detección: es CI-6, no CE-3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>R1166</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Comentario» → [Excluir CI-6] Plataforma de videovigilancia con detección y seguimiento de vehículos; muestra ejemplos de incidentes, pero no reporta métricas de detección.</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Coherente con CI-6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>R1185</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Entorno» → No reportado</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>No clasifica las imágenes por tipo de vía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>R1202</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Corregido «Partición» → Prueba independiente</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Separación por sesiones de conducción.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
           <t>R1214</t>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="C95" s="4" t="inlineStr">
         <is>
           <t>Corregido «Partición» → No reportada</t>
         </is>
       </c>
-      <c r="D81" s="4" t="inlineStr">
+      <c r="D95" s="4" t="inlineStr">
         <is>
           <t>No informa proporciones ni criterio de división.</t>
         </is>

</xml_diff>